<commit_message>
Add Yesterday filter tab, reorder period tabs, permanently remove 250 Rs test sale, and improve delete sync
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,51 +447,95 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790808573942_ktuq</v>
+        <v>sale_1790839031379</v>
       </c>
       <c r="B2" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C2" t="str">
-        <v>03182642966</v>
+        <v>+92 340 7317084</v>
       </c>
       <c r="D2" t="str">
-        <v>Ali Ahmed</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>Abd114@kuromee.com</v>
+        <v>Nord9@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="K2" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-09-30T22:49:33.942Z</v>
+        <v>2026-10-01T07:17:11.379Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sale_1790838846301</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>3085352533</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G3" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>800</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-11-29</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2 Devices</v>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Filter pending KPI stats, tab counts, and pending list by selected period
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,95 +447,139 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790891345201_z6tu</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C2" t="str">
-        <v>+92 340 7317084</v>
+        <v>dssds</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>Sgsg</v>
       </c>
       <c r="H2" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-01T21:49:05.201Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790839031379</v>
       </c>
       <c r="B3" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C3" t="str">
-        <v>3085352533</v>
+        <v>+92 340 7317084</v>
       </c>
       <c r="D3" t="str">
         <v/>
       </c>
       <c r="E3" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Nord9@kuromee.com</v>
+      </c>
+      <c r="H3" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>500</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-10-01T07:17:11.379Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>sale_1790838846301</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>3085352533</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
         <v>Surfshark</v>
       </c>
-      <c r="F3" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="G3" t="str">
+      <c r="F4" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G4" t="str">
         <v>abd149@kuromee.com</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H4" t="str">
         <v>2 Months (60 Days)</v>
       </c>
-      <c r="I3">
+      <c r="I4">
         <v>2</v>
       </c>
-      <c r="J3">
+      <c r="J4">
         <v>800</v>
       </c>
-      <c r="K3" t="str">
+      <c r="K4" t="str">
         <v>Pending</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L4" t="str">
         <v>2026-11-29</v>
       </c>
-      <c r="M3" t="str">
+      <c r="M4" t="str">
         <v>2 Devices</v>
       </c>
-      <c r="N3" t="str">
+      <c r="N4" t="str">
         <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix cross-device sync: prevent restore from overwriting PIN, fix verify-pin server sync, and permanently purge test entries
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,139 +447,95 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790891345201_z6tu</v>
+        <v>sale_1790839031379</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C2" t="str">
-        <v>dssds</v>
+        <v>+92 340 7317084</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>Sgsg</v>
+        <v>Nord9@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-01T21:49:05.201Z</v>
+        <v>2026-10-01T07:17:11.379Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790838846301</v>
       </c>
       <c r="B3" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C3" t="str">
-        <v>+92 340 7317084</v>
+        <v>3085352533</v>
       </c>
       <c r="D3" t="str">
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F3" t="str">
         <v>Shared</v>
       </c>
       <c r="G3" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H3" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="K3" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2 Devices</v>
       </c>
       <c r="N3" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>sale_1790838846301</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-10-01</v>
-      </c>
-      <c r="C4" t="str">
-        <v>3085352533</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="G4" t="str">
-        <v>abd149@kuromee.com</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2 Months (60 Days)</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>800</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="L4" t="str">
-        <v>2026-11-29</v>
-      </c>
-      <c r="M4" t="str">
-        <v>2 Devices</v>
-      </c>
-      <c r="N4" t="str">
         <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restore all 19 sales and 4 expenses in database and ledger
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,57 +447,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790889578017</v>
       </c>
       <c r="B2" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C2" t="str">
-        <v>+92 340 7317084</v>
+        <v>03000000000</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-01T20:59:38.017Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790888324786</v>
       </c>
       <c r="B3" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C3" t="str">
-        <v>3085352533</v>
+        <v>3424112890 - 232013</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -512,37 +512,785 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H3" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>250</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L3" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-10-01T20:58:44.786Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>sale_1790871288858</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>+92 336 6331621</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G4" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H4" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1200</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>2026-10-01T16:14:48.858Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>sale_1790871264002</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>+98 901 603 6081</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G5" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H5" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>500</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-10-01T16:14:24.002Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>sale_1790868862060</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>+92 341 9010662</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G6" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1000</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L6" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-10-01T15:34:22.075Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>sale_1790864924575</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>+92 313 6762957</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G7" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H7" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>500</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v>2026-10-01T14:28:44.576Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>sale_1790864890520</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C8" t="str">
+        <v>3166729551</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G8" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H8" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8">
+        <v>600</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L8" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v>2026-10-01T14:28:10.520Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>sale_1790862744178</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>+92 317 0295905</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G9" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H9" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I9">
+        <v>3</v>
+      </c>
+      <c r="J9">
+        <v>600</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>2026-10-01T13:52:24.178Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>sale_1790861118501</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C10" t="str">
+        <v>+92 344 4643148</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G10" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H10" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="J10">
+        <v>500</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L10" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v>2026-10-01T13:25:18.501Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>sale_1790853314445</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C11" t="str">
+        <v>+92 302 7283125</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H11" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>750</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L11" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M11" t="str">
+        <v>vukdsas@apricity.tech  masuk123</v>
+      </c>
+      <c r="N11" t="str">
+        <v>2026-10-01T11:15:14.445Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>sale_1790852538710</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C12" t="str">
+        <v>+92 325 1501138</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H12" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>1000</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L12" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v>2026-10-01T11:02:18.710Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>sale_1790852373016</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C13" t="str">
+        <v>+92 301 7890066</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G13" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H13" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1500</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L13" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v>2026-10-01T10:59:33.016Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>sale_1790850006978</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C14" t="str">
+        <v>+92 342 4112890-534389</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G14" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H14" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>200</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L14" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v>2026-10-01T10:20:06.978Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>sale_1790849948623</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C15" t="str">
+        <v>+92 349 6363398</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G15" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H15" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>250</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L15" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v>2026-10-01T10:19:08.625Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>sale_1790844774858</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C16" t="str">
+        <v>03035587360</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Not applicable</v>
+      </c>
+      <c r="H16" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="I16">
+        <v>18</v>
+      </c>
+      <c r="J16">
+        <v>500</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L16" t="str">
+        <v>2028-03-23</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v>2026-10-01T08:52:54.860Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>sale_1790841917101</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C17" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G17" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H17" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>500</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L17" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v>2026-10-01T08:05:17.101Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>sale_1790890880426_oulk</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C18" t="str">
+        <v>3336677666</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G18" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H18" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>250</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v>2026-10-01T21:41:20.426Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>sale_1790839031379</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C19" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Nord9@kuromee.com</v>
+      </c>
+      <c r="H19" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+      <c r="J19">
+        <v>500</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L19" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v>2026-10-01T07:17:11.379Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>sale_1790838846301</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C20" t="str">
+        <v>3085352533</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G20" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H20" t="str">
         <v>2 Months (60 Days)</v>
       </c>
-      <c r="I3">
+      <c r="I20">
         <v>2</v>
       </c>
-      <c r="J3">
+      <c r="J20">
         <v>800</v>
       </c>
-      <c r="K3" t="str">
+      <c r="K20" t="str">
         <v>Pending</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L20" t="str">
         <v>2026-11-29</v>
       </c>
-      <c r="M3" t="str">
+      <c r="M20" t="str">
         <v>2 Devices</v>
       </c>
-      <c r="N3" t="str">
+      <c r="N20" t="str">
         <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N20"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -584,9 +1332,69 @@
         <v>2026-09-30T23:28:01.227Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>exp_1790889252470</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Surfshark/Nord Paid</v>
+      </c>
+      <c r="E3">
+        <v>1600</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-10-01T21:14:12.470Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>exp_1790888895390</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Capcut padmahastuti3@akunku.site|masuk123</v>
+      </c>
+      <c r="E4">
+        <v>350</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-10-01T21:08:15.390Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>exp_1790865001001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Capcut Account For Luxury online Store   vukdsas@apricity.tech:masuk123</v>
+      </c>
+      <c r="E5">
+        <v>350</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-10-01T14:30:01.001Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restore all 29 sales, 4 expenses, and full ledger database
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,57 +447,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790889578017</v>
+        <v>sale_1790839031379</v>
       </c>
       <c r="B2" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C2" t="str">
-        <v>03000000000</v>
+        <v>+92 340 7317084</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>Nord9@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-29</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-01T20:59:38.017Z</v>
+        <v>2026-10-01T07:17:11.379Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790888324786</v>
+        <v>sale_1790838846301</v>
       </c>
       <c r="B3" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C3" t="str">
-        <v>3424112890 - 232013</v>
+        <v>3085352533</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -512,48 +512,48 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H3" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="K3" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2 Devices</v>
       </c>
       <c r="N3" t="str">
-        <v>2026-10-01T20:58:44.786Z</v>
+        <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sale_1790871288858</v>
+        <v>sale_1790890878620</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C4" t="str">
-        <v>+92 336 6331621</v>
+        <v>3336677666</v>
       </c>
       <c r="D4" t="str">
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F4" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G4" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H4" t="str">
         <v>1 Month (30 Days)</v>
@@ -562,86 +562,86 @@
         <v>1</v>
       </c>
       <c r="J4">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="K4" t="str">
         <v>Paid</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M4" t="str">
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-10-01T16:14:48.858Z</v>
+        <v>2026-10-01T21:41:18.621Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>sale_1790871264002</v>
+        <v>sale_1790889330982</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C5" t="str">
-        <v>+98 901 603 6081</v>
+        <v>+92 333 7180888</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F5" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G5" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H5" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K5" t="str">
         <v>Paid</v>
       </c>
       <c r="L5" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M5" t="str">
         <v/>
       </c>
       <c r="N5" t="str">
-        <v>2026-10-01T16:14:24.002Z</v>
+        <v>2026-10-01T21:15:30.982Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>sale_1790868862060</v>
+        <v>sale_1790889206450</v>
       </c>
       <c r="B6" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C6" t="str">
-        <v>+92 341 9010662</v>
+        <v>447348556756 - 2 Devices</v>
       </c>
       <c r="D6" t="str">
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F6" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G6" t="str">
-        <v>NA</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H6" t="str">
         <v>1 Month (30 Days)</v>
@@ -650,10 +650,10 @@
         <v>1</v>
       </c>
       <c r="J6">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="K6" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L6" t="str">
         <v>2026-10-30</v>
@@ -662,206 +662,206 @@
         <v/>
       </c>
       <c r="N6" t="str">
-        <v>2026-10-01T15:34:22.075Z</v>
+        <v>2026-10-01T21:13:26.450Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sale_1790864924575</v>
+        <v>sale_1790889149110</v>
       </c>
       <c r="B7" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C7" t="str">
-        <v>+92 313 6762957</v>
+        <v>3716928959</v>
       </c>
       <c r="D7" t="str">
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F7" t="str">
         <v>Shared</v>
       </c>
       <c r="G7" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H7" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K7" t="str">
         <v>Paid</v>
       </c>
       <c r="L7" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M7" t="str">
         <v/>
       </c>
       <c r="N7" t="str">
-        <v>2026-10-01T14:28:44.576Z</v>
+        <v>2026-10-01T21:12:29.110Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>sale_1790864890520</v>
+        <v>sale_1790889019841</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C8" t="str">
-        <v>3166729551</v>
+        <v>+92 324 3715759</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F8" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G8" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H8" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="K8" t="str">
         <v>Paid</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M8" t="str">
         <v/>
       </c>
       <c r="N8" t="str">
-        <v>2026-10-01T14:28:10.520Z</v>
+        <v>2026-10-01T21:10:19.841Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sale_1790862744178</v>
+        <v>sale_1790888980587</v>
       </c>
       <c r="B9" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C9" t="str">
-        <v>+92 317 0295905</v>
+        <v>+92 337 8569003</v>
       </c>
       <c r="D9" t="str">
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>Nord</v>
+        <v>CapCut</v>
       </c>
       <c r="F9" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G9" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>padmahastuti3@akunku.site|masuk123</v>
       </c>
       <c r="H9" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="K9" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L9" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M9" t="str">
         <v/>
       </c>
       <c r="N9" t="str">
-        <v>2026-10-01T13:52:24.178Z</v>
+        <v>2026-10-01T21:09:40.587Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>sale_1790861118501</v>
+        <v>sale_1790888790593</v>
       </c>
       <c r="B10" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C10" t="str">
-        <v>+92 344 4643148</v>
+        <v>+92 318 8934627</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F10" t="str">
         <v>Shared</v>
       </c>
       <c r="G10" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H10" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="K10" t="str">
         <v>Paid</v>
       </c>
       <c r="L10" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M10" t="str">
         <v/>
       </c>
       <c r="N10" t="str">
-        <v>2026-10-01T13:25:18.501Z</v>
+        <v>2026-10-01T21:06:30.593Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sale_1790853314445</v>
+        <v>sale_1790888748366</v>
       </c>
       <c r="B11" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C11" t="str">
-        <v>+92 302 7283125</v>
+        <v>3121600439</v>
       </c>
       <c r="D11" t="str">
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F11" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G11" t="str">
-        <v>NA</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H11" t="str">
         <v>1 Month (30 Days)</v>
@@ -870,42 +870,42 @@
         <v>1</v>
       </c>
       <c r="J11">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="K11" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L11" t="str">
         <v>2026-10-30</v>
       </c>
       <c r="M11" t="str">
-        <v>vukdsas@apricity.tech  masuk123</v>
+        <v/>
       </c>
       <c r="N11" t="str">
-        <v>2026-10-01T11:15:14.445Z</v>
+        <v>2026-10-01T21:05:48.366Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sale_1790852538710</v>
+        <v>sale_1790888549930</v>
       </c>
       <c r="B12" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C12" t="str">
-        <v>+92 325 1501138</v>
+        <v>3148646368</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F12" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G12" t="str">
-        <v>N/A</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H12" t="str">
         <v>1 Month (30 Days)</v>
@@ -914,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="J12">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="K12" t="str">
         <v>Paid</v>
@@ -926,62 +926,62 @@
         <v/>
       </c>
       <c r="N12" t="str">
-        <v>2026-10-01T11:02:18.710Z</v>
+        <v>2026-10-01T21:02:29.930Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sale_1790852373016</v>
+        <v>sale_1790888489800</v>
       </c>
       <c r="B13" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C13" t="str">
-        <v>+92 301 7890066</v>
+        <v>3043943233 - 2 devices</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F13" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G13" t="str">
-        <v>N/A</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H13" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J13">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="K13" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L13" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>Payment 5 Oct</v>
       </c>
       <c r="N13" t="str">
-        <v>2026-10-01T10:59:33.016Z</v>
+        <v>2026-10-01T21:01:29.800Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sale_1790850006978</v>
+        <v>sale_1790888426010</v>
       </c>
       <c r="B14" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C14" t="str">
-        <v>+92 342 4112890-534389</v>
+        <v>3125698180</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -996,36 +996,36 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H14" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="K14" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L14" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>Payment Sunday 4 Oct</v>
       </c>
       <c r="N14" t="str">
-        <v>2026-10-01T10:20:06.978Z</v>
+        <v>2026-10-01T21:00:26.011Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sale_1790849948623</v>
+        <v>sale_1790888378017</v>
       </c>
       <c r="B15" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C15" t="str">
-        <v>+92 349 6363398</v>
+        <v>3208546164</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -1040,250 +1040,690 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H15" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J15">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="K15" t="str">
         <v>Paid</v>
       </c>
       <c r="L15" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M15" t="str">
         <v/>
       </c>
       <c r="N15" t="str">
-        <v>2026-10-01T10:19:08.625Z</v>
+        <v>2026-10-01T20:59:38.017Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>sale_1790844774858</v>
+        <v>sale_1790888324786</v>
       </c>
       <c r="B16" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C16" t="str">
-        <v>03035587360</v>
+        <v>3424112890 - 232013</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Gemini Pro</v>
+        <v>Surfshark</v>
       </c>
       <c r="F16" t="str">
         <v>Shared</v>
       </c>
       <c r="G16" t="str">
-        <v>Not applicable</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H16" t="str">
-        <v>18 Months (540 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I16">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K16" t="str">
         <v>Paid</v>
       </c>
       <c r="L16" t="str">
-        <v>2028-03-23</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M16" t="str">
         <v/>
       </c>
       <c r="N16" t="str">
-        <v>2026-10-01T08:52:54.860Z</v>
+        <v>2026-10-01T20:58:44.786Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>sale_1790841917101</v>
+        <v>sale_1790871288858</v>
       </c>
       <c r="B17" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C17" t="str">
-        <v>+92 340 7317084</v>
+        <v>+92 336 6331621</v>
       </c>
       <c r="D17" t="str">
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F17" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G17" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H17" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="K17" t="str">
         <v>Paid</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M17" t="str">
         <v/>
       </c>
       <c r="N17" t="str">
-        <v>2026-10-01T08:05:17.101Z</v>
+        <v>2026-10-01T16:14:48.858Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>sale_1790890880426_oulk</v>
+        <v>sale_1790871264002</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-01</v>
       </c>
       <c r="C18" t="str">
-        <v>3336677666</v>
+        <v>+98 901 603 6081</v>
       </c>
       <c r="D18" t="str">
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F18" t="str">
         <v>Shared</v>
       </c>
       <c r="G18" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H18" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J18">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="K18" t="str">
         <v>Paid</v>
       </c>
       <c r="L18" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M18" t="str">
         <v/>
       </c>
       <c r="N18" t="str">
-        <v>2026-10-01T21:41:20.426Z</v>
+        <v>2026-10-01T16:14:24.002Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790868862060</v>
       </c>
       <c r="B19" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C19" t="str">
-        <v>+92 340 7317084</v>
+        <v>+92 341 9010662</v>
       </c>
       <c r="D19" t="str">
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F19" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G19" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H19" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K19" t="str">
         <v>Paid</v>
       </c>
       <c r="L19" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M19" t="str">
         <v/>
       </c>
       <c r="N19" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-01T15:34:22.075Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790864924575</v>
       </c>
       <c r="B20" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C20" t="str">
-        <v>3085352533</v>
+        <v>+92 313 6762957</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G20" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H20" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I20">
+        <v>3</v>
+      </c>
+      <c r="J20">
+        <v>500</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v>2026-10-01T14:28:44.576Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>sale_1790864890520</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C21" t="str">
+        <v>3166729551</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
         <v>Surfshark</v>
       </c>
-      <c r="F20" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="G20" t="str">
+      <c r="F21" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G21" t="str">
         <v>abd149@kuromee.com</v>
       </c>
-      <c r="H20" t="str">
-        <v>2 Months (60 Days)</v>
-      </c>
-      <c r="I20">
-        <v>2</v>
-      </c>
-      <c r="J20">
-        <v>800</v>
-      </c>
-      <c r="K20" t="str">
+      <c r="H21" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>600</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L21" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v>2026-10-01T14:28:10.520Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>sale_1790862744178</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C22" t="str">
+        <v>+92 317 0295905</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G22" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H22" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I22">
+        <v>3</v>
+      </c>
+      <c r="J22">
+        <v>600</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L22" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v>2026-10-01T13:52:24.178Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>sale_1790861118501</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C23" t="str">
+        <v>+92 344 4643148</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G23" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H23" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>500</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L23" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v>2026-10-01T13:25:18.501Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>sale_1790853314445</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C24" t="str">
+        <v>+92 302 7283125</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G24" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H24" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24">
+        <v>750</v>
+      </c>
+      <c r="K24" t="str">
         <v>Pending</v>
       </c>
-      <c r="L20" t="str">
-        <v>2026-11-29</v>
-      </c>
-      <c r="M20" t="str">
-        <v>2 Devices</v>
-      </c>
-      <c r="N20" t="str">
-        <v>2026-10-01T07:14:06.302Z</v>
+      <c r="L24" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M24" t="str">
+        <v>vukdsas@apricity.tech  masuk123</v>
+      </c>
+      <c r="N24" t="str">
+        <v>2026-10-01T11:15:14.445Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>sale_1790852538710</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C25" t="str">
+        <v>+92 325 1501138</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H25" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+      <c r="J25">
+        <v>1000</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L25" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v>2026-10-01T11:02:18.710Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>sale_1790852373016</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C26" t="str">
+        <v>+92 301 7890066</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G26" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H26" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+      <c r="J26">
+        <v>1500</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L26" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v>2026-10-01T10:59:33.016Z</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>sale_1790850006978</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C27" t="str">
+        <v>+92 342 4112890-534389</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G27" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H27" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I27">
+        <v>1</v>
+      </c>
+      <c r="J27">
+        <v>200</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L27" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v>2026-10-01T10:20:06.978Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>sale_1790849948623</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C28" t="str">
+        <v>+92 349 6363398</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G28" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H28" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="J28">
+        <v>250</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L28" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v>2026-10-01T10:19:08.625Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>sale_1790844774858</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C29" t="str">
+        <v>03035587360</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Not applicable</v>
+      </c>
+      <c r="H29" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="I29">
+        <v>18</v>
+      </c>
+      <c r="J29">
+        <v>500</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L29" t="str">
+        <v>2028-03-23</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v>2026-10-01T08:52:54.860Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>sale_1790841917101</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C30" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G30" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H30" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+      <c r="J30">
+        <v>500</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L30" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v>2026-10-01T08:05:17.101Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restore all 39 sales, protect against data wipe on refresh, and enable non-destructive cross-device sync
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,57 +447,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790934819273</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C2" t="str">
-        <v>+92 340 7317084</v>
+        <v>3362088885</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-02T09:53:39.274Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790934132194</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C3" t="str">
-        <v>3085352533</v>
+        <v>3171626906</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -509,39 +509,39 @@
         <v>Shared</v>
       </c>
       <c r="G3" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H3" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="K3" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M3" t="str">
-        <v>2 Devices</v>
+        <v/>
       </c>
       <c r="N3" t="str">
-        <v>2026-10-01T07:14:06.302Z</v>
+        <v>2026-10-02T09:42:12.194Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sale_1790890878620</v>
+        <v>sale_1790929984076</v>
       </c>
       <c r="B4" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C4" t="str">
-        <v>3336677666</v>
+        <v>3425091286</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -574,18 +574,18 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-10-01T21:41:18.621Z</v>
+        <v>2026-10-02T08:33:04.076Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>sale_1790889330982</v>
+        <v>sale_1790928896570</v>
       </c>
       <c r="B5" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C5" t="str">
-        <v>+92 333 7180888</v>
+        <v>+92 335 9333443</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -594,7 +594,7 @@
         <v>Muse AI</v>
       </c>
       <c r="F5" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G5" t="str">
         <v>NA</v>
@@ -606,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="J5">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="K5" t="str">
         <v>Paid</v>
@@ -618,18 +618,18 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v>2026-10-01T21:15:30.982Z</v>
+        <v>2026-10-02T08:14:56.570Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>sale_1790889206450</v>
+        <v>sale_1790927823366</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C6" t="str">
-        <v>447348556756 - 2 Devices</v>
+        <v>3424112890 - 178132</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -641,7 +641,7 @@
         <v>Shared</v>
       </c>
       <c r="G6" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H6" t="str">
         <v>1 Month (30 Days)</v>
@@ -650,30 +650,30 @@
         <v>1</v>
       </c>
       <c r="J6">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="K6" t="str">
         <v>Pending</v>
       </c>
       <c r="L6" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M6" t="str">
         <v/>
       </c>
       <c r="N6" t="str">
-        <v>2026-10-01T21:13:26.450Z</v>
+        <v>2026-10-02T07:57:03.366Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sale_1790889149110</v>
+        <v>sale_1790927720999</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C7" t="str">
-        <v>3716928959</v>
+        <v>3355060692</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -685,95 +685,95 @@
         <v>Shared</v>
       </c>
       <c r="G7" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H7" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="K7" t="str">
         <v>Paid</v>
       </c>
       <c r="L7" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M7" t="str">
         <v/>
       </c>
       <c r="N7" t="str">
-        <v>2026-10-01T21:12:29.110Z</v>
+        <v>2026-10-02T07:55:20.999Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>sale_1790889019841</v>
+        <v>sale_1790927520048</v>
       </c>
       <c r="B8" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C8" t="str">
-        <v>+92 324 3715759</v>
+        <v>3237432065</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F8" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G8" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H8" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="K8" t="str">
         <v>Paid</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M8" t="str">
         <v/>
       </c>
       <c r="N8" t="str">
-        <v>2026-10-01T21:10:19.841Z</v>
+        <v>2026-10-02T07:52:00.048Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sale_1790888980587</v>
+        <v>sale_1790927399372</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C9" t="str">
-        <v>+92 337 8569003</v>
+        <v>3226763778</v>
       </c>
       <c r="D9" t="str">
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F9" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G9" t="str">
-        <v>padmahastuti3@akunku.site|masuk123</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H9" t="str">
         <v>1 Month (30 Days)</v>
@@ -782,42 +782,42 @@
         <v>1</v>
       </c>
       <c r="J9">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="K9" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L9" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M9" t="str">
         <v/>
       </c>
       <c r="N9" t="str">
-        <v>2026-10-01T21:09:40.587Z</v>
+        <v>2026-10-02T07:49:59.372Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>sale_1790888790593</v>
+        <v>sale_1790927194315</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C10" t="str">
-        <v>+92 318 8934627</v>
+        <v>3087182016</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F10" t="str">
         <v>Shared</v>
       </c>
       <c r="G10" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H10" t="str">
         <v>1 Month (30 Days)</v>
@@ -826,30 +826,30 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="K10" t="str">
         <v>Paid</v>
       </c>
       <c r="L10" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M10" t="str">
         <v/>
       </c>
       <c r="N10" t="str">
-        <v>2026-10-01T21:06:30.593Z</v>
+        <v>2026-10-02T07:46:34.315Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sale_1790888748366</v>
+        <v>sale_1790926790421</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C11" t="str">
-        <v>3121600439</v>
+        <v>3424112890 - 161547</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -861,7 +861,7 @@
         <v>Shared</v>
       </c>
       <c r="G11" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H11" t="str">
         <v>1 Month (30 Days)</v>
@@ -870,30 +870,30 @@
         <v>1</v>
       </c>
       <c r="J11">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="K11" t="str">
         <v>Paid</v>
       </c>
       <c r="L11" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M11" t="str">
         <v/>
       </c>
       <c r="N11" t="str">
-        <v>2026-10-01T21:05:48.366Z</v>
+        <v>2026-10-02T07:39:50.422Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sale_1790888549930</v>
+        <v>sale_1790890878620</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C12" t="str">
-        <v>3148646368</v>
+        <v>3336677666</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -905,7 +905,7 @@
         <v>Shared</v>
       </c>
       <c r="G12" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H12" t="str">
         <v>1 Month (30 Days)</v>
@@ -914,118 +914,118 @@
         <v>1</v>
       </c>
       <c r="J12">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="K12" t="str">
         <v>Paid</v>
       </c>
       <c r="L12" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M12" t="str">
         <v/>
       </c>
       <c r="N12" t="str">
-        <v>2026-10-01T21:02:29.930Z</v>
+        <v>2026-10-01T21:41:18.621Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sale_1790888489800</v>
+        <v>sale_1790889330982</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C13" t="str">
-        <v>3043943233 - 2 devices</v>
+        <v>+92 333 7180888</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F13" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G13" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H13" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J13">
         <v>1000</v>
       </c>
       <c r="K13" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L13" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M13" t="str">
-        <v>Payment 5 Oct</v>
+        <v/>
       </c>
       <c r="N13" t="str">
-        <v>2026-10-01T21:01:29.800Z</v>
+        <v>2026-10-01T21:15:30.982Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sale_1790888426010</v>
+        <v>sale_1790889019841</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C14" t="str">
-        <v>3125698180</v>
+        <v>+92 324 3715759</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F14" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G14" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H14" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="K14" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L14" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M14" t="str">
-        <v>Payment Sunday 4 Oct</v>
+        <v/>
       </c>
       <c r="N14" t="str">
-        <v>2026-10-01T21:00:26.011Z</v>
+        <v>2026-10-01T21:10:19.841Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sale_1790888378017</v>
+        <v>sale_1790889206450</v>
       </c>
       <c r="B15" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C15" t="str">
-        <v>3208546164</v>
+        <v>447348556756 - 2 Devices</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -1040,36 +1040,36 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H15" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J15">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="K15" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L15" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M15" t="str">
         <v/>
       </c>
       <c r="N15" t="str">
-        <v>2026-10-01T20:59:38.017Z</v>
+        <v>2026-10-01T21:13:26.450Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>sale_1790888324786</v>
+        <v>sale_1790889149110</v>
       </c>
       <c r="B16" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C16" t="str">
-        <v>3424112890 - 232013</v>
+        <v>3716928959</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -1084,48 +1084,48 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H16" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="K16" t="str">
         <v>Paid</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M16" t="str">
         <v/>
       </c>
       <c r="N16" t="str">
-        <v>2026-10-01T20:58:44.786Z</v>
+        <v>2026-10-01T21:12:29.110Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>sale_1790871288858</v>
+        <v>sale_1790888980587</v>
       </c>
       <c r="B17" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C17" t="str">
-        <v>+92 336 6331621</v>
+        <v>+92 337 8569003</v>
       </c>
       <c r="D17" t="str">
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>Muse AI</v>
+        <v>CapCut</v>
       </c>
       <c r="F17" t="str">
         <v>Private</v>
       </c>
       <c r="G17" t="str">
-        <v>NA</v>
+        <v>padmahastuti3@akunku.site|masuk123</v>
       </c>
       <c r="H17" t="str">
         <v>1 Month (30 Days)</v>
@@ -1134,10 +1134,10 @@
         <v>1</v>
       </c>
       <c r="J17">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="K17" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L17" t="str">
         <v>2026-10-30</v>
@@ -1146,74 +1146,74 @@
         <v/>
       </c>
       <c r="N17" t="str">
-        <v>2026-10-01T16:14:48.858Z</v>
+        <v>2026-10-01T21:09:40.587Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>sale_1790871264002</v>
+        <v>sale_1790888790593</v>
       </c>
       <c r="B18" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C18" t="str">
-        <v>+98 901 603 6081</v>
+        <v>+92 318 8934627</v>
       </c>
       <c r="D18" t="str">
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F18" t="str">
         <v>Shared</v>
       </c>
       <c r="G18" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H18" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="K18" t="str">
         <v>Paid</v>
       </c>
       <c r="L18" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M18" t="str">
         <v/>
       </c>
       <c r="N18" t="str">
-        <v>2026-10-01T16:14:24.002Z</v>
+        <v>2026-10-01T21:06:30.593Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>sale_1790868862060</v>
+        <v>sale_1790888748366</v>
       </c>
       <c r="B19" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C19" t="str">
-        <v>+92 341 9010662</v>
+        <v>3121600439</v>
       </c>
       <c r="D19" t="str">
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F19" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G19" t="str">
-        <v>NA</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H19" t="str">
         <v>1 Month (30 Days)</v>
@@ -1222,7 +1222,7 @@
         <v>1</v>
       </c>
       <c r="J19">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="K19" t="str">
         <v>Paid</v>
@@ -1234,62 +1234,62 @@
         <v/>
       </c>
       <c r="N19" t="str">
-        <v>2026-10-01T15:34:22.075Z</v>
+        <v>2026-10-01T21:05:48.366Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>sale_1790864924575</v>
+        <v>sale_1790888549930</v>
       </c>
       <c r="B20" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C20" t="str">
-        <v>+92 313 6762957</v>
+        <v>3148646368</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F20" t="str">
         <v>Shared</v>
       </c>
       <c r="G20" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H20" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="K20" t="str">
         <v>Paid</v>
       </c>
       <c r="L20" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M20" t="str">
         <v/>
       </c>
       <c r="N20" t="str">
-        <v>2026-10-01T14:28:44.576Z</v>
+        <v>2026-10-01T21:02:29.930Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>sale_1790864890520</v>
+        <v>sale_1790888489800</v>
       </c>
       <c r="B21" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C21" t="str">
-        <v>3166729551</v>
+        <v>3043943233 - 2 devices</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -1310,130 +1310,130 @@
         <v>3</v>
       </c>
       <c r="J21">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="K21" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L21" t="str">
         <v>2026-12-29</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>Payment 5 Oct</v>
       </c>
       <c r="N21" t="str">
-        <v>2026-10-01T14:28:10.520Z</v>
+        <v>2026-10-01T21:01:29.800Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>sale_1790862744178</v>
+        <v>sale_1790888426010</v>
       </c>
       <c r="B22" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C22" t="str">
-        <v>+92 317 0295905</v>
+        <v>3125698180</v>
       </c>
       <c r="D22" t="str">
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F22" t="str">
         <v>Shared</v>
       </c>
       <c r="G22" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H22" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J22">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="K22" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L22" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>Payment Sunday 4 Oct</v>
       </c>
       <c r="N22" t="str">
-        <v>2026-10-01T13:52:24.178Z</v>
+        <v>2026-10-01T21:00:26.011Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>sale_1790861118501</v>
+        <v>sale_1790888378017</v>
       </c>
       <c r="B23" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C23" t="str">
-        <v>+92 344 4643148</v>
+        <v>3208546164</v>
       </c>
       <c r="D23" t="str">
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F23" t="str">
         <v>Shared</v>
       </c>
       <c r="G23" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H23" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K23" t="str">
         <v>Paid</v>
       </c>
       <c r="L23" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v>2026-10-01T13:25:18.501Z</v>
+        <v>2026-10-01T20:59:38.017Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>sale_1790853314445</v>
+        <v>sale_1790888324786</v>
       </c>
       <c r="B24" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C24" t="str">
-        <v>+92 302 7283125</v>
+        <v>3424112890 - 232013</v>
       </c>
       <c r="D24" t="str">
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F24" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G24" t="str">
-        <v>NA</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H24" t="str">
         <v>1 Month (30 Days)</v>
@@ -1442,30 +1442,30 @@
         <v>1</v>
       </c>
       <c r="J24">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="K24" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L24" t="str">
         <v>2026-10-30</v>
       </c>
       <c r="M24" t="str">
-        <v>vukdsas@apricity.tech  masuk123</v>
+        <v/>
       </c>
       <c r="N24" t="str">
-        <v>2026-10-01T11:15:14.445Z</v>
+        <v>2026-10-01T20:58:44.786Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>sale_1790852538710</v>
+        <v>sale_1790871288858</v>
       </c>
       <c r="B25" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C25" t="str">
-        <v>+92 325 1501138</v>
+        <v>+92 336 6331621</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -1477,7 +1477,7 @@
         <v>Private</v>
       </c>
       <c r="G25" t="str">
-        <v>N/A</v>
+        <v>NA</v>
       </c>
       <c r="H25" t="str">
         <v>1 Month (30 Days)</v>
@@ -1486,7 +1486,7 @@
         <v>1</v>
       </c>
       <c r="J25">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="K25" t="str">
         <v>Paid</v>
@@ -1498,74 +1498,74 @@
         <v/>
       </c>
       <c r="N25" t="str">
-        <v>2026-10-01T11:02:18.710Z</v>
+        <v>2026-10-01T16:14:48.858Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>sale_1790852373016</v>
+        <v>sale_1790871264002</v>
       </c>
       <c r="B26" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C26" t="str">
-        <v>+92 301 7890066</v>
+        <v>+98 901 603 6081</v>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>Muse AI</v>
+        <v>Nord</v>
       </c>
       <c r="F26" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G26" t="str">
-        <v>N/A</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H26" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J26">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="K26" t="str">
         <v>Paid</v>
       </c>
       <c r="L26" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M26" t="str">
         <v/>
       </c>
       <c r="N26" t="str">
-        <v>2026-10-01T10:59:33.016Z</v>
+        <v>2026-10-01T16:14:24.002Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>sale_1790850006978</v>
+        <v>sale_1790868862060</v>
       </c>
       <c r="B27" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C27" t="str">
-        <v>+92 342 4112890-534389</v>
+        <v>+92 341 9010662</v>
       </c>
       <c r="D27" t="str">
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F27" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G27" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H27" t="str">
         <v>1 Month (30 Days)</v>
@@ -1574,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="J27">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="K27" t="str">
         <v>Paid</v>
@@ -1586,106 +1586,106 @@
         <v/>
       </c>
       <c r="N27" t="str">
-        <v>2026-10-01T10:20:06.978Z</v>
+        <v>2026-10-01T15:34:22.075Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>sale_1790849948623</v>
+        <v>sale_1790864924575</v>
       </c>
       <c r="B28" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C28" t="str">
-        <v>+92 349 6363398</v>
+        <v>+92 313 6762957</v>
       </c>
       <c r="D28" t="str">
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F28" t="str">
         <v>Shared</v>
       </c>
       <c r="G28" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H28" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J28">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="K28" t="str">
         <v>Paid</v>
       </c>
       <c r="L28" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>2026-10-01T10:19:08.625Z</v>
+        <v>2026-10-01T14:28:44.576Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>sale_1790844774858</v>
+        <v>sale_1790864890520</v>
       </c>
       <c r="B29" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C29" t="str">
-        <v>03035587360</v>
+        <v>3166729551</v>
       </c>
       <c r="D29" t="str">
         <v/>
       </c>
       <c r="E29" t="str">
-        <v>Gemini Pro</v>
+        <v>Surfshark</v>
       </c>
       <c r="F29" t="str">
         <v>Shared</v>
       </c>
       <c r="G29" t="str">
-        <v>Not applicable</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H29" t="str">
-        <v>18 Months (540 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I29">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="K29" t="str">
         <v>Paid</v>
       </c>
       <c r="L29" t="str">
-        <v>2028-03-23</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M29" t="str">
         <v/>
       </c>
       <c r="N29" t="str">
-        <v>2026-10-01T08:52:54.860Z</v>
+        <v>2026-10-01T14:28:10.520Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>sale_1790841917101</v>
+        <v>sale_1790862744178</v>
       </c>
       <c r="B30" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C30" t="str">
-        <v>+92 340 7317084</v>
+        <v>+92 317 0295905</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>3</v>
       </c>
       <c r="J30">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="K30" t="str">
         <v>Paid</v>
@@ -1718,12 +1718,452 @@
         <v/>
       </c>
       <c r="N30" t="str">
+        <v>2026-10-01T13:52:24.178Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>sale_1790861118501</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C31" t="str">
+        <v>+92 344 4643148</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G31" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H31" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I31">
+        <v>3</v>
+      </c>
+      <c r="J31">
+        <v>500</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L31" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v>2026-10-01T13:25:18.501Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>sale_1790853314445</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C32" t="str">
+        <v>+92 302 7283125</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G32" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H32" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <v>750</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L32" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M32" t="str">
+        <v>vukdsas@apricity.tech  masuk123</v>
+      </c>
+      <c r="N32" t="str">
+        <v>2026-10-01T11:15:14.445Z</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>sale_1790852538710</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C33" t="str">
+        <v>+92 325 1501138</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G33" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H33" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>1000</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L33" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v>2026-10-01T11:02:18.710Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>sale_1790852373016</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C34" t="str">
+        <v>+92 301 7890066</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G34" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H34" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>1500</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L34" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v>2026-10-01T10:59:33.016Z</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>sale_1790850006978</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C35" t="str">
+        <v>+92 342 4112890-534389</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G35" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H35" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>200</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L35" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v>2026-10-01T10:20:06.978Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>sale_1790849948623</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C36" t="str">
+        <v>+92 349 6363398</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G36" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H36" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36">
+        <v>250</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L36" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v>2026-10-01T10:19:08.625Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>sale_1790844774858</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C37" t="str">
+        <v>03035587360</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Not applicable</v>
+      </c>
+      <c r="H37" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="I37">
+        <v>18</v>
+      </c>
+      <c r="J37">
+        <v>500</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L37" t="str">
+        <v>2028-03-23</v>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v>2026-10-01T08:52:54.860Z</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>sale_1790841917101</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C38" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G38" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H38" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I38">
+        <v>3</v>
+      </c>
+      <c r="J38">
+        <v>500</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L38" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
         <v>2026-10-01T08:05:17.101Z</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>sale_1790839031379</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C39" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Nord9@kuromee.com</v>
+      </c>
+      <c r="H39" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I39">
+        <v>3</v>
+      </c>
+      <c r="J39">
+        <v>500</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L39" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v>2026-10-01T07:17:11.379Z</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>sale_1790838846301</v>
+      </c>
+      <c r="B40" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C40" t="str">
+        <v>3085352533</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G40" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H40" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="I40">
+        <v>2</v>
+      </c>
+      <c r="J40">
+        <v>800</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L40" t="str">
+        <v>2026-11-29</v>
+      </c>
+      <c r="M40" t="str">
+        <v>2 Devices</v>
+      </c>
+      <c r="N40" t="str">
+        <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restore all 54 sales & 6 expenses, add instant auto-save without refresh, and enable real-time bidirectional sync
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,57 +447,57 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790934819273</v>
+        <v>sale_1790972901458</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C2" t="str">
-        <v>3362088885</v>
+        <v>+92 333 3707266</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F2" t="str">
         <v>Shared</v>
       </c>
       <c r="G2" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H2" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-31</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-02T09:53:39.274Z</v>
+        <v>2026-10-02T20:28:21.458Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790934132194</v>
+        <v>sale_1790971693632</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C3" t="str">
-        <v>3171626906</v>
+        <v>3038522190</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -512,36 +512,36 @@
         <v>abd150@kuromee.com</v>
       </c>
       <c r="H3" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="K3" t="str">
         <v>Paid</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-01</v>
       </c>
       <c r="M3" t="str">
         <v/>
       </c>
       <c r="N3" t="str">
-        <v>2026-10-02T09:42:12.194Z</v>
+        <v>2026-10-02T20:08:13.632Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sale_1790929984076</v>
+        <v>sale_1790967903952</v>
       </c>
       <c r="B4" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C4" t="str">
-        <v>3425091286</v>
+        <v>3452401920</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -556,48 +556,48 @@
         <v>abd150@kuromee.com</v>
       </c>
       <c r="H4" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="K4" t="str">
         <v>Paid</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M4" t="str">
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-10-02T08:33:04.076Z</v>
+        <v>2026-10-02T19:05:03.952Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>sale_1790928896570</v>
+        <v>sale_1790966446338</v>
       </c>
       <c r="B5" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C5" t="str">
-        <v>+92 335 9333443</v>
+        <v>3162936885</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F5" t="str">
         <v>Shared</v>
       </c>
       <c r="G5" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H5" t="str">
         <v>1 Month (30 Days)</v>
@@ -606,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="J5">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="K5" t="str">
         <v>Paid</v>
@@ -618,18 +618,18 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v>2026-10-02T08:14:56.570Z</v>
+        <v>2026-10-02T18:40:46.338Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>sale_1790927823366</v>
+        <v>sale_1790964840039</v>
       </c>
       <c r="B6" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C6" t="str">
-        <v>3424112890 - 178132</v>
+        <v>3068258151</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -650,10 +650,10 @@
         <v>1</v>
       </c>
       <c r="J6">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="K6" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L6" t="str">
         <v>2026-10-31</v>
@@ -662,30 +662,30 @@
         <v/>
       </c>
       <c r="N6" t="str">
-        <v>2026-10-02T07:57:03.366Z</v>
+        <v>2026-10-02T18:14:00.039Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sale_1790927720999</v>
+        <v>sale_1790964482569</v>
       </c>
       <c r="B7" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C7" t="str">
-        <v>3355060692</v>
+        <v>+92 334 7132394</v>
       </c>
       <c r="D7" t="str">
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F7" t="str">
         <v>Shared</v>
       </c>
       <c r="G7" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H7" t="str">
         <v>1 Month (30 Days)</v>
@@ -694,7 +694,7 @@
         <v>1</v>
       </c>
       <c r="J7">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="K7" t="str">
         <v>Paid</v>
@@ -706,62 +706,62 @@
         <v/>
       </c>
       <c r="N7" t="str">
-        <v>2026-10-02T07:55:20.999Z</v>
+        <v>2026-10-02T18:08:02.570Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>sale_1790927520048</v>
+        <v>sale_1790964455099</v>
       </c>
       <c r="B8" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C8" t="str">
-        <v>3237432065</v>
+        <v>+92 318 8934627</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F8" t="str">
         <v>Shared</v>
       </c>
       <c r="G8" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H8" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="K8" t="str">
         <v>Paid</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-11-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M8" t="str">
         <v/>
       </c>
       <c r="N8" t="str">
-        <v>2026-10-02T07:52:00.048Z</v>
+        <v>2026-10-02T18:07:35.099Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sale_1790927399372</v>
+        <v>sale_1790955121286</v>
       </c>
       <c r="B9" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C9" t="str">
-        <v>3226763778</v>
+        <v>3424112890 - 810813</v>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -782,10 +782,10 @@
         <v>1</v>
       </c>
       <c r="J9">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="K9" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L9" t="str">
         <v>2026-10-31</v>
@@ -794,30 +794,30 @@
         <v/>
       </c>
       <c r="N9" t="str">
-        <v>2026-10-02T07:49:59.372Z</v>
+        <v>2026-10-02T15:32:01.286Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>sale_1790927194315</v>
+        <v>sale_1790954315594</v>
       </c>
       <c r="B10" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C10" t="str">
-        <v>3087182016</v>
+        <v>+92 339 8895511</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F10" t="str">
         <v>Shared</v>
       </c>
       <c r="G10" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H10" t="str">
         <v>1 Month (30 Days)</v>
@@ -826,7 +826,7 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>250</v>
+        <v>1200</v>
       </c>
       <c r="K10" t="str">
         <v>Paid</v>
@@ -838,118 +838,118 @@
         <v/>
       </c>
       <c r="N10" t="str">
-        <v>2026-10-02T07:46:34.315Z</v>
+        <v>2026-10-02T15:18:35.594Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sale_1790926790421</v>
+        <v>sale_1790946519871</v>
       </c>
       <c r="B11" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C11" t="str">
-        <v>3424112890 - 161547</v>
+        <v>+92 337 4695990</v>
       </c>
       <c r="D11" t="str">
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F11" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G11" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H11" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>200</v>
+        <v>1300</v>
       </c>
       <c r="K11" t="str">
         <v>Paid</v>
       </c>
       <c r="L11" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-30</v>
       </c>
       <c r="M11" t="str">
         <v/>
       </c>
       <c r="N11" t="str">
-        <v>2026-10-02T07:39:50.422Z</v>
+        <v>2026-10-02T13:08:39.871Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sale_1790890878620</v>
+        <v>sale_1790946456992</v>
       </c>
       <c r="B12" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C12" t="str">
-        <v>3336677666</v>
+        <v>+92 310 8747472</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F12" t="str">
         <v>Shared</v>
       </c>
       <c r="G12" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>nor8@kuromee.com</v>
       </c>
       <c r="H12" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>6 Months (180 Days)</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J12">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="K12" t="str">
         <v>Paid</v>
       </c>
       <c r="L12" t="str">
-        <v>2026-10-31</v>
+        <v>2027-03-30</v>
       </c>
       <c r="M12" t="str">
         <v/>
       </c>
       <c r="N12" t="str">
-        <v>2026-10-01T21:41:18.621Z</v>
+        <v>2026-10-02T13:07:36.993Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sale_1790889330982</v>
+        <v>sale_1790941037212</v>
       </c>
       <c r="B13" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C13" t="str">
-        <v>+92 333 7180888</v>
+        <v>30474552522</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F13" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G13" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H13" t="str">
         <v>1 Month (30 Days)</v>
@@ -958,7 +958,7 @@
         <v>1</v>
       </c>
       <c r="J13">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="K13" t="str">
         <v>Paid</v>
@@ -970,74 +970,74 @@
         <v/>
       </c>
       <c r="N13" t="str">
-        <v>2026-10-01T21:15:30.982Z</v>
+        <v>2026-10-02T11:37:17.212Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sale_1790889019841</v>
+        <v>sale_1790940354053</v>
       </c>
       <c r="B14" t="str">
         <v>2026-10-02</v>
       </c>
       <c r="C14" t="str">
-        <v>+92 324 3715759</v>
+        <v>+92 333 5598645</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F14" t="str">
         <v>Private</v>
       </c>
       <c r="G14" t="str">
-        <v>NA</v>
+        <v>alissaturner822@gmail.com</v>
       </c>
       <c r="H14" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="K14" t="str">
         <v>Paid</v>
       </c>
       <c r="L14" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M14" t="str">
         <v/>
       </c>
       <c r="N14" t="str">
-        <v>2026-10-01T21:10:19.841Z</v>
+        <v>2026-10-02T11:25:54.053Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sale_1790889206450</v>
+        <v>sale_1790939431495</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C15" t="str">
-        <v>447348556756 - 2 Devices</v>
+        <v>+92 301 2553778</v>
       </c>
       <c r="D15" t="str">
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F15" t="str">
         <v>Shared</v>
       </c>
       <c r="G15" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H15" t="str">
         <v>1 Month (30 Days)</v>
@@ -1046,30 +1046,30 @@
         <v>1</v>
       </c>
       <c r="J15">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="K15" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L15" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M15" t="str">
         <v/>
       </c>
       <c r="N15" t="str">
-        <v>2026-10-01T21:13:26.450Z</v>
+        <v>2026-10-02T11:10:31.495Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>sale_1790889149110</v>
+        <v>sale_1790936221232</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C16" t="str">
-        <v>3716928959</v>
+        <v>3362088885</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -1081,51 +1081,51 @@
         <v>Shared</v>
       </c>
       <c r="G16" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H16" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="K16" t="str">
         <v>Paid</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M16" t="str">
         <v/>
       </c>
       <c r="N16" t="str">
-        <v>2026-10-01T21:12:29.110Z</v>
+        <v>2026-10-02T10:17:01.232Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>sale_1790888980587</v>
+        <v>sale_1790934819273</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C17" t="str">
-        <v>+92 337 8569003</v>
+        <v>3362088885</v>
       </c>
       <c r="D17" t="str">
         <v/>
       </c>
       <c r="E17" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F17" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G17" t="str">
-        <v>padmahastuti3@akunku.site|masuk123</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H17" t="str">
         <v>1 Month (30 Days)</v>
@@ -1134,42 +1134,42 @@
         <v>1</v>
       </c>
       <c r="J17">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="K17" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M17" t="str">
         <v/>
       </c>
       <c r="N17" t="str">
-        <v>2026-10-01T21:09:40.587Z</v>
+        <v>2026-10-02T09:53:39.274Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>sale_1790888790593</v>
+        <v>sale_1790934132194</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C18" t="str">
-        <v>+92 318 8934627</v>
+        <v>3171626906</v>
       </c>
       <c r="D18" t="str">
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F18" t="str">
         <v>Shared</v>
       </c>
       <c r="G18" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H18" t="str">
         <v>1 Month (30 Days)</v>
@@ -1178,30 +1178,30 @@
         <v>1</v>
       </c>
       <c r="J18">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="K18" t="str">
         <v>Paid</v>
       </c>
       <c r="L18" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M18" t="str">
         <v/>
       </c>
       <c r="N18" t="str">
-        <v>2026-10-01T21:06:30.593Z</v>
+        <v>2026-10-02T09:42:12.194Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>sale_1790888748366</v>
+        <v>sale_1790929984076</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C19" t="str">
-        <v>3121600439</v>
+        <v>3425091286</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -1213,7 +1213,7 @@
         <v>Shared</v>
       </c>
       <c r="G19" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H19" t="str">
         <v>1 Month (30 Days)</v>
@@ -1228,36 +1228,36 @@
         <v>Paid</v>
       </c>
       <c r="L19" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M19" t="str">
         <v/>
       </c>
       <c r="N19" t="str">
-        <v>2026-10-01T21:05:48.366Z</v>
+        <v>2026-10-02T08:33:04.076Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>sale_1790888549930</v>
+        <v>sale_1790928896570</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C20" t="str">
-        <v>3148646368</v>
+        <v>+92 335 9333443</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F20" t="str">
         <v>Shared</v>
       </c>
       <c r="G20" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H20" t="str">
         <v>1 Month (30 Days)</v>
@@ -1266,30 +1266,30 @@
         <v>1</v>
       </c>
       <c r="J20">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="K20" t="str">
         <v>Paid</v>
       </c>
       <c r="L20" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M20" t="str">
         <v/>
       </c>
       <c r="N20" t="str">
-        <v>2026-10-01T21:02:29.930Z</v>
+        <v>2026-10-02T08:14:56.570Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>sale_1790888489800</v>
+        <v>sale_1790927823366</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C21" t="str">
-        <v>3043943233 - 2 devices</v>
+        <v>3424112890 - 178132</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -1301,39 +1301,39 @@
         <v>Shared</v>
       </c>
       <c r="G21" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H21" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J21">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="K21" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L21" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M21" t="str">
-        <v>Payment 5 Oct</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>2026-10-01T21:01:29.800Z</v>
+        <v>2026-10-02T07:57:03.366Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>sale_1790888426010</v>
+        <v>sale_1790927720999</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C22" t="str">
-        <v>3125698180</v>
+        <v>3355060692</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -1345,39 +1345,39 @@
         <v>Shared</v>
       </c>
       <c r="G22" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H22" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="K22" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L22" t="str">
-        <v>2026-11-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M22" t="str">
-        <v>Payment Sunday 4 Oct</v>
+        <v/>
       </c>
       <c r="N22" t="str">
-        <v>2026-10-01T21:00:26.011Z</v>
+        <v>2026-10-02T07:55:20.999Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>sale_1790888378017</v>
+        <v>sale_1790927520048</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C23" t="str">
-        <v>3208546164</v>
+        <v>3237432065</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -1389,7 +1389,7 @@
         <v>Shared</v>
       </c>
       <c r="G23" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H23" t="str">
         <v>2 Months (60 Days)</v>
@@ -1404,24 +1404,24 @@
         <v>Paid</v>
       </c>
       <c r="L23" t="str">
-        <v>2026-11-29</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v>2026-10-01T20:59:38.017Z</v>
+        <v>2026-10-02T07:52:00.048Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>sale_1790888324786</v>
+        <v>sale_1790927399372</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C24" t="str">
-        <v>3424112890 - 232013</v>
+        <v>3226763778</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -1433,7 +1433,7 @@
         <v>Shared</v>
       </c>
       <c r="G24" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H24" t="str">
         <v>1 Month (30 Days)</v>
@@ -1448,36 +1448,36 @@
         <v>Paid</v>
       </c>
       <c r="L24" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M24" t="str">
         <v/>
       </c>
       <c r="N24" t="str">
-        <v>2026-10-01T20:58:44.786Z</v>
+        <v>2026-10-02T07:49:59.372Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>sale_1790871288858</v>
+        <v>sale_1790927194315</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C25" t="str">
-        <v>+92 336 6331621</v>
+        <v>3087182016</v>
       </c>
       <c r="D25" t="str">
         <v/>
       </c>
       <c r="E25" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F25" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G25" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H25" t="str">
         <v>1 Month (30 Days)</v>
@@ -1486,86 +1486,86 @@
         <v>1</v>
       </c>
       <c r="J25">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="K25" t="str">
         <v>Paid</v>
       </c>
       <c r="L25" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M25" t="str">
         <v/>
       </c>
       <c r="N25" t="str">
-        <v>2026-10-01T16:14:48.858Z</v>
+        <v>2026-10-02T07:46:34.315Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>sale_1790871264002</v>
+        <v>sale_1790926790421</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C26" t="str">
-        <v>+98 901 603 6081</v>
+        <v>3424112890 - 161547</v>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F26" t="str">
         <v>Shared</v>
       </c>
       <c r="G26" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H26" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="K26" t="str">
         <v>Paid</v>
       </c>
       <c r="L26" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M26" t="str">
         <v/>
       </c>
       <c r="N26" t="str">
-        <v>2026-10-01T16:14:24.002Z</v>
+        <v>2026-10-02T07:39:50.422Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>sale_1790868862060</v>
+        <v>sale_1790890878620</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C27" t="str">
-        <v>+92 341 9010662</v>
+        <v>3336677666</v>
       </c>
       <c r="D27" t="str">
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F27" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G27" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H27" t="str">
         <v>1 Month (30 Days)</v>
@@ -1574,206 +1574,206 @@
         <v>1</v>
       </c>
       <c r="J27">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="K27" t="str">
         <v>Paid</v>
       </c>
       <c r="L27" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M27" t="str">
         <v/>
       </c>
       <c r="N27" t="str">
-        <v>2026-10-01T15:34:22.075Z</v>
+        <v>2026-10-01T21:41:18.621Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>sale_1790864924575</v>
+        <v>sale_1790889330982</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C28" t="str">
-        <v>+92 313 6762957</v>
+        <v>+92 333 7180888</v>
       </c>
       <c r="D28" t="str">
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F28" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G28" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H28" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I28">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K28" t="str">
         <v>Paid</v>
       </c>
       <c r="L28" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>2026-10-01T14:28:44.576Z</v>
+        <v>2026-10-01T21:15:30.982Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>sale_1790864890520</v>
+        <v>sale_1790889019841</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C29" t="str">
-        <v>3166729551</v>
+        <v>+92 324 3715759</v>
       </c>
       <c r="D29" t="str">
         <v/>
       </c>
       <c r="E29" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F29" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G29" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H29" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J29">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="K29" t="str">
         <v>Paid</v>
       </c>
       <c r="L29" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M29" t="str">
         <v/>
       </c>
       <c r="N29" t="str">
-        <v>2026-10-01T14:28:10.520Z</v>
+        <v>2026-10-01T21:10:19.841Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>sale_1790862744178</v>
+        <v>sale_1790889206450</v>
       </c>
       <c r="B30" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C30" t="str">
-        <v>+92 317 0295905</v>
+        <v>447348556756 - 2 Devices</v>
       </c>
       <c r="D30" t="str">
         <v/>
       </c>
       <c r="E30" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F30" t="str">
         <v>Shared</v>
       </c>
       <c r="G30" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H30" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J30">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="K30" t="str">
         <v>Paid</v>
       </c>
       <c r="L30" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M30" t="str">
         <v/>
       </c>
       <c r="N30" t="str">
-        <v>2026-10-01T13:52:24.178Z</v>
+        <v>2026-10-01T21:13:26.450Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>sale_1790861118501</v>
+        <v>sale_1790889149110</v>
       </c>
       <c r="B31" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C31" t="str">
-        <v>+92 344 4643148</v>
+        <v>3716928959</v>
       </c>
       <c r="D31" t="str">
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F31" t="str">
         <v>Shared</v>
       </c>
       <c r="G31" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H31" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J31">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K31" t="str">
         <v>Paid</v>
       </c>
       <c r="L31" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
-        <v>2026-10-01T13:25:18.501Z</v>
+        <v>2026-10-01T21:12:29.110Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>sale_1790853314445</v>
+        <v>sale_1790888980587</v>
       </c>
       <c r="B32" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C32" t="str">
-        <v>+92 302 7283125</v>
+        <v>+92 337 8569003</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -1785,7 +1785,7 @@
         <v>Private</v>
       </c>
       <c r="G32" t="str">
-        <v>NA</v>
+        <v>padmahastuti3@akunku.site|masuk123</v>
       </c>
       <c r="H32" t="str">
         <v>1 Month (30 Days)</v>
@@ -1803,21 +1803,21 @@
         <v>2026-10-30</v>
       </c>
       <c r="M32" t="str">
-        <v>vukdsas@apricity.tech  masuk123</v>
+        <v/>
       </c>
       <c r="N32" t="str">
-        <v>2026-10-01T11:15:14.445Z</v>
+        <v>2026-10-01T21:09:40.587Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>sale_1790852538710</v>
+        <v>sale_1790888790593</v>
       </c>
       <c r="B33" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C33" t="str">
-        <v>+92 325 1501138</v>
+        <v>+92 318 8934627</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -1826,10 +1826,10 @@
         <v>Muse AI</v>
       </c>
       <c r="F33" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G33" t="str">
-        <v>N/A</v>
+        <v>NA</v>
       </c>
       <c r="H33" t="str">
         <v>1 Month (30 Days)</v>
@@ -1838,7 +1838,7 @@
         <v>1</v>
       </c>
       <c r="J33">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="K33" t="str">
         <v>Paid</v>
@@ -1850,30 +1850,30 @@
         <v/>
       </c>
       <c r="N33" t="str">
-        <v>2026-10-01T11:02:18.710Z</v>
+        <v>2026-10-01T21:06:30.593Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>sale_1790852373016</v>
+        <v>sale_1790888748366</v>
       </c>
       <c r="B34" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C34" t="str">
-        <v>+92 301 7890066</v>
+        <v>3121600439</v>
       </c>
       <c r="D34" t="str">
         <v/>
       </c>
       <c r="E34" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F34" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G34" t="str">
-        <v>N/A</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H34" t="str">
         <v>1 Month (30 Days)</v>
@@ -1882,7 +1882,7 @@
         <v>1</v>
       </c>
       <c r="J34">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="K34" t="str">
         <v>Paid</v>
@@ -1894,18 +1894,18 @@
         <v/>
       </c>
       <c r="N34" t="str">
-        <v>2026-10-01T10:59:33.016Z</v>
+        <v>2026-10-01T21:05:48.366Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>sale_1790850006978</v>
+        <v>sale_1790888549930</v>
       </c>
       <c r="B35" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C35" t="str">
-        <v>+92 342 4112890-534389</v>
+        <v>3148646368</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -1938,18 +1938,18 @@
         <v/>
       </c>
       <c r="N35" t="str">
-        <v>2026-10-01T10:20:06.978Z</v>
+        <v>2026-10-01T21:02:29.930Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>sale_1790849948623</v>
+        <v>sale_1790888489800</v>
       </c>
       <c r="B36" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C36" t="str">
-        <v>+92 349 6363398</v>
+        <v>3043943233 - 2 devices</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -1964,213 +1964,873 @@
         <v>abd149@kuromee.com</v>
       </c>
       <c r="H36" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="K36" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L36" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-29</v>
       </c>
       <c r="M36" t="str">
-        <v/>
+        <v>Payment 5 Oct</v>
       </c>
       <c r="N36" t="str">
-        <v>2026-10-01T10:19:08.625Z</v>
+        <v>2026-10-01T21:01:29.800Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>sale_1790844774858</v>
+        <v>sale_1790888426010</v>
       </c>
       <c r="B37" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C37" t="str">
-        <v>03035587360</v>
+        <v>3125698180</v>
       </c>
       <c r="D37" t="str">
         <v/>
       </c>
       <c r="E37" t="str">
-        <v>Gemini Pro</v>
+        <v>Surfshark</v>
       </c>
       <c r="F37" t="str">
         <v>Shared</v>
       </c>
       <c r="G37" t="str">
-        <v>Not applicable</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H37" t="str">
-        <v>18 Months (540 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I37">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J37">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K37" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L37" t="str">
-        <v>2028-03-23</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M37" t="str">
-        <v/>
+        <v>Payment Sunday 4 Oct</v>
       </c>
       <c r="N37" t="str">
-        <v>2026-10-01T08:52:54.860Z</v>
+        <v>2026-10-01T21:00:26.011Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>sale_1790841917101</v>
+        <v>sale_1790888378017</v>
       </c>
       <c r="B38" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C38" t="str">
-        <v>+92 340 7317084</v>
+        <v>3208546164</v>
       </c>
       <c r="D38" t="str">
         <v/>
       </c>
       <c r="E38" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F38" t="str">
         <v>Shared</v>
       </c>
       <c r="G38" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H38" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J38">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="K38" t="str">
         <v>Paid</v>
       </c>
       <c r="L38" t="str">
-        <v>2026-12-29</v>
+        <v>2026-11-29</v>
       </c>
       <c r="M38" t="str">
         <v/>
       </c>
       <c r="N38" t="str">
-        <v>2026-10-01T08:05:17.101Z</v>
+        <v>2026-10-01T20:59:38.017Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790888324786</v>
       </c>
       <c r="B39" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C39" t="str">
-        <v>+92 340 7317084</v>
+        <v>3424112890 - 232013</v>
       </c>
       <c r="D39" t="str">
         <v/>
       </c>
       <c r="E39" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F39" t="str">
         <v>Shared</v>
       </c>
       <c r="G39" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>abd149@kuromee.com</v>
       </c>
       <c r="H39" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I39">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J39">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K39" t="str">
         <v>Paid</v>
       </c>
       <c r="L39" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="M39" t="str">
         <v/>
       </c>
       <c r="N39" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-01T20:58:44.786Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790871288858</v>
       </c>
       <c r="B40" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C40" t="str">
+        <v>+92 336 6331621</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G40" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H40" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40">
+        <v>1200</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L40" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v>2026-10-01T16:14:48.858Z</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>sale_1790871264002</v>
+      </c>
+      <c r="B41" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C41" t="str">
+        <v>+98 901 603 6081</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G41" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H41" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I41">
+        <v>3</v>
+      </c>
+      <c r="J41">
+        <v>500</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L41" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v>2026-10-01T16:14:24.002Z</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>sale_1790868862060</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C42" t="str">
+        <v>+92 341 9010662</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G42" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H42" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="J42">
+        <v>1000</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L42" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v>2026-10-01T15:34:22.075Z</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>sale_1790864924575</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C43" t="str">
+        <v>+92 313 6762957</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G43" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H43" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I43">
+        <v>3</v>
+      </c>
+      <c r="J43">
+        <v>500</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L43" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M43" t="str">
+        <v/>
+      </c>
+      <c r="N43" t="str">
+        <v>2026-10-01T14:28:44.576Z</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>sale_1790864890520</v>
+      </c>
+      <c r="B44" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C44" t="str">
+        <v>3166729551</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G44" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H44" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>600</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L44" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M44" t="str">
+        <v/>
+      </c>
+      <c r="N44" t="str">
+        <v>2026-10-01T14:28:10.520Z</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>sale_1790862744178</v>
+      </c>
+      <c r="B45" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C45" t="str">
+        <v>+92 317 0295905</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G45" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H45" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I45">
+        <v>3</v>
+      </c>
+      <c r="J45">
+        <v>600</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L45" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M45" t="str">
+        <v/>
+      </c>
+      <c r="N45" t="str">
+        <v>2026-10-01T13:52:24.178Z</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>sale_1790861118501</v>
+      </c>
+      <c r="B46" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C46" t="str">
+        <v>+92 344 4643148</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G46" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H46" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I46">
+        <v>3</v>
+      </c>
+      <c r="J46">
+        <v>500</v>
+      </c>
+      <c r="K46" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L46" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M46" t="str">
+        <v/>
+      </c>
+      <c r="N46" t="str">
+        <v>2026-10-01T13:25:18.501Z</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>sale_1790853314445</v>
+      </c>
+      <c r="B47" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C47" t="str">
+        <v>+92 302 7283125</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G47" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H47" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I47">
+        <v>1</v>
+      </c>
+      <c r="J47">
+        <v>750</v>
+      </c>
+      <c r="K47" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L47" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M47" t="str">
+        <v>vukdsas@apricity.tech  masuk123</v>
+      </c>
+      <c r="N47" t="str">
+        <v>2026-10-01T11:15:14.445Z</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>sale_1790852538710</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C48" t="str">
+        <v>+92 325 1501138</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G48" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H48" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+      <c r="J48">
+        <v>1000</v>
+      </c>
+      <c r="K48" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L48" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M48" t="str">
+        <v/>
+      </c>
+      <c r="N48" t="str">
+        <v>2026-10-01T11:02:18.710Z</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>sale_1790852373016</v>
+      </c>
+      <c r="B49" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C49" t="str">
+        <v>+92 301 7890066</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G49" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H49" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
+      <c r="J49">
+        <v>1500</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L49" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M49" t="str">
+        <v/>
+      </c>
+      <c r="N49" t="str">
+        <v>2026-10-01T10:59:33.016Z</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>sale_1790850006978</v>
+      </c>
+      <c r="B50" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C50" t="str">
+        <v>+92 342 4112890-534389</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G50" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H50" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50">
+        <v>200</v>
+      </c>
+      <c r="K50" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L50" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M50" t="str">
+        <v/>
+      </c>
+      <c r="N50" t="str">
+        <v>2026-10-01T10:20:06.978Z</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>sale_1790849948623</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C51" t="str">
+        <v>+92 349 6363398</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G51" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H51" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51">
+        <v>250</v>
+      </c>
+      <c r="K51" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L51" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M51" t="str">
+        <v/>
+      </c>
+      <c r="N51" t="str">
+        <v>2026-10-01T10:19:08.625Z</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>sale_1790844774858</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C52" t="str">
+        <v>03035587360</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Not applicable</v>
+      </c>
+      <c r="H52" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="I52">
+        <v>18</v>
+      </c>
+      <c r="J52">
+        <v>500</v>
+      </c>
+      <c r="K52" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L52" t="str">
+        <v>2028-03-23</v>
+      </c>
+      <c r="M52" t="str">
+        <v/>
+      </c>
+      <c r="N52" t="str">
+        <v>2026-10-01T08:52:54.860Z</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>sale_1790841917101</v>
+      </c>
+      <c r="B53" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C53" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G53" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H53" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I53">
+        <v>3</v>
+      </c>
+      <c r="J53">
+        <v>500</v>
+      </c>
+      <c r="K53" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L53" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M53" t="str">
+        <v/>
+      </c>
+      <c r="N53" t="str">
+        <v>2026-10-01T08:05:17.101Z</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>sale_1790839031379</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C54" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Nord9@kuromee.com</v>
+      </c>
+      <c r="H54" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I54">
+        <v>3</v>
+      </c>
+      <c r="J54">
+        <v>500</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L54" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M54" t="str">
+        <v/>
+      </c>
+      <c r="N54" t="str">
+        <v>2026-10-01T07:17:11.379Z</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>sale_1790838846301</v>
+      </c>
+      <c r="B55" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C55" t="str">
         <v>3085352533</v>
       </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
-      <c r="E40" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="F40" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="G40" t="str">
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G55" t="str">
         <v>abd149@kuromee.com</v>
       </c>
-      <c r="H40" t="str">
+      <c r="H55" t="str">
         <v>2 Months (60 Days)</v>
       </c>
-      <c r="I40">
+      <c r="I55">
         <v>2</v>
       </c>
-      <c r="J40">
+      <c r="J55">
         <v>800</v>
       </c>
-      <c r="K40" t="str">
+      <c r="K55" t="str">
         <v>Pending</v>
       </c>
-      <c r="L40" t="str">
+      <c r="L55" t="str">
         <v>2026-11-29</v>
       </c>
-      <c r="M40" t="str">
+      <c r="M55" t="str">
         <v>2 Devices</v>
       </c>
-      <c r="N40" t="str">
+      <c r="N55" t="str">
         <v>2026-10-01T07:14:06.302Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N55"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2194,47 +2854,47 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>exp_1790810881227_1bq9</v>
+        <v>exp_1790946533413</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C2" t="str">
-        <v>Meta Ads</v>
+        <v>Vendor Purchasing</v>
       </c>
       <c r="D2" t="str">
-        <v>Meta Ads Campaign</v>
+        <v>Nord purchasing</v>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>850</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-30T23:28:01.227Z</v>
+        <v>2026-10-02T13:08:53.414Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>exp_1790889252470</v>
+        <v>exp_1790940392222</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C3" t="str">
         <v>Vendor Purchasing</v>
       </c>
       <c r="D3" t="str">
-        <v>Surfshark/Nord Paid</v>
+        <v>alissaturner822@gmail.com   Surfshark Private Payment</v>
       </c>
       <c r="E3">
-        <v>1600</v>
+        <v>750</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-10-01T21:14:12.470Z</v>
+        <v>2026-10-02T11:26:32.222Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>exp_1790888895390</v>
+        <v>exp_1790889252470</v>
       </c>
       <c r="B4" t="str">
         <v>2026-10-01</v>
@@ -2243,18 +2903,18 @@
         <v>Vendor Purchasing</v>
       </c>
       <c r="D4" t="str">
-        <v>Capcut padmahastuti3@akunku.site|masuk123</v>
+        <v>Surfshark/Nord Paid</v>
       </c>
       <c r="E4">
-        <v>350</v>
+        <v>1600</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-10-01T21:08:15.390Z</v>
+        <v>2026-10-01T21:14:12.470Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>exp_1790865001001</v>
+        <v>exp_1790888895390</v>
       </c>
       <c r="B5" t="str">
         <v>2026-10-01</v>
@@ -2263,18 +2923,58 @@
         <v>Vendor Purchasing</v>
       </c>
       <c r="D5" t="str">
-        <v>Capcut Account For Luxury online Store   vukdsas@apricity.tech:masuk123</v>
+        <v>Capcut padmahastuti3@akunku.site|masuk123</v>
       </c>
       <c r="E5">
         <v>350</v>
       </c>
       <c r="F5" t="str">
+        <v>2026-10-01T21:08:15.390Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>exp_1790865001001</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Capcut Account For Luxury online Store   vukdsas@apricity.tech:masuk123</v>
+      </c>
+      <c r="E6">
+        <v>350</v>
+      </c>
+      <c r="F6" t="str">
         <v>2026-10-01T14:30:01.001Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>exp_1790810881227_1bq9</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Meta Ads</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Meta Ads Campaign</v>
+      </c>
+      <c r="E7">
+        <v>500</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-30T23:28:01.227Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Auto-save and real-time sync for all settings, product catalog, pricing plans, and PIN changes
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -2981,7 +2981,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3289,9 +3289,26 @@
         <v>500</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Test Product</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>1M</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Protect Reset/Start Fresh action with Master Password Sad12345@
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -2981,7 +2981,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3289,26 +3289,9 @@
         <v>500</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Test Product</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" t="str">
-        <v>1M</v>
-      </c>
-      <c r="E19">
-        <v>100</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix cross-device real-time sync between PC and mobile: await Cloud KV on serverless, add API no-cache headers, add fetch timeout and queueing, and sync latest records
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -5,7 +5,6 @@
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
     <sheet name="Expenses" sheetId="2" r:id="rId2"/>
-    <sheet name="Products" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:N89"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,189 +446,189 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>sale_1790972901458</v>
+        <v>sale_1791205614503</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C2" t="str">
-        <v>+92 333 3707266</v>
+        <v>+92 344 9282193</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F2" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G2" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H2" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K2" t="str">
         <v>Paid</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-12-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M2" t="str">
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-10-02T20:28:21.458Z</v>
+        <v>2026-10-05T13:06:54.503Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>sale_1790971693632</v>
+        <v>sale_1791205520863</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C3" t="str">
-        <v>3038522190</v>
+        <v>+92 336 2088885</v>
       </c>
       <c r="D3" t="str">
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>Surfshark</v>
+        <v>CapCut</v>
       </c>
       <c r="F3" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G3" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>baktionopradana64@akunku.site  masuk123  qaoyxh@apricity.tech  masuk123</v>
       </c>
       <c r="H3" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (25 Days)</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>400</v>
+        <v>1100</v>
       </c>
       <c r="K3" t="str">
         <v>Paid</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-12-01</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2 Capcut</v>
       </c>
       <c r="N3" t="str">
-        <v>2026-10-02T20:08:13.632Z</v>
+        <v>2026-10-05T13:05:20.863Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sale_1790967903952</v>
+        <v>sale_1791205472496</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C4" t="str">
-        <v>3452401920</v>
+        <v>+92 300 2689698</v>
       </c>
       <c r="D4" t="str">
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F4" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G4" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H4" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="K4" t="str">
         <v>Paid</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-11-30</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M4" t="str">
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-10-02T19:05:03.952Z</v>
+        <v>2026-10-05T13:04:32.497Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>sale_1790966446338</v>
+        <v>sale_1791193680484</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C5" t="str">
-        <v>3162936885</v>
+        <v>+92 341 5984031</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F5" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G5" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H5" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="K5" t="str">
         <v>Paid</v>
       </c>
       <c r="L5" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M5" t="str">
         <v/>
       </c>
       <c r="N5" t="str">
-        <v>2026-10-02T18:40:46.338Z</v>
+        <v>2026-10-05T09:48:00.484Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>sale_1790964840039</v>
+        <v>sale_1791191267464</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C6" t="str">
-        <v>3068258151</v>
+        <v>3317376555</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -641,7 +640,7 @@
         <v>Shared</v>
       </c>
       <c r="G6" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H6" t="str">
         <v>1 Month (30 Days)</v>
@@ -656,80 +655,80 @@
         <v>Paid</v>
       </c>
       <c r="L6" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M6" t="str">
         <v/>
       </c>
       <c r="N6" t="str">
-        <v>2026-10-02T18:14:00.039Z</v>
+        <v>2026-10-05T09:07:47.464Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sale_1790964482569</v>
+        <v>sale_1791187749963</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C7" t="str">
-        <v>+92 334 7132394</v>
+        <v>+92 326 4813460</v>
       </c>
       <c r="D7" t="str">
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Muse AI</v>
+        <v>Nord</v>
       </c>
       <c r="F7" t="str">
         <v>Shared</v>
       </c>
       <c r="G7" t="str">
-        <v>NA</v>
+        <v>nord10@kuromee.com</v>
       </c>
       <c r="H7" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="K7" t="str">
         <v>Paid</v>
       </c>
       <c r="L7" t="str">
-        <v>2026-10-31</v>
+        <v>2027-01-02</v>
       </c>
       <c r="M7" t="str">
         <v/>
       </c>
       <c r="N7" t="str">
-        <v>2026-10-02T18:08:02.570Z</v>
+        <v>2026-10-05T08:09:09.963Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>sale_1790964455099</v>
+        <v>sale_1791187520074</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C8" t="str">
-        <v>+92 318 8934627</v>
+        <v>3005130980</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F8" t="str">
         <v>Shared</v>
       </c>
       <c r="G8" t="str">
-        <v>NA</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H8" t="str">
         <v>1 Month (30 Days)</v>
@@ -738,30 +737,30 @@
         <v>1</v>
       </c>
       <c r="J8">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="K8" t="str">
         <v>Paid</v>
       </c>
       <c r="L8" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M8" t="str">
         <v/>
       </c>
       <c r="N8" t="str">
-        <v>2026-10-02T18:07:35.099Z</v>
+        <v>2026-10-05T08:05:20.074Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>sale_1790955121286</v>
+        <v>sale_1791187470511</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C9" t="str">
-        <v>3424112890 - 810813</v>
+        <v>3443570380</v>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -773,7 +772,7 @@
         <v>Shared</v>
       </c>
       <c r="G9" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H9" t="str">
         <v>1 Month (30 Days)</v>
@@ -788,74 +787,74 @@
         <v>Pending</v>
       </c>
       <c r="L9" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M9" t="str">
         <v/>
       </c>
       <c r="N9" t="str">
-        <v>2026-10-02T15:32:01.286Z</v>
+        <v>2026-10-05T08:04:30.511Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>sale_1790954315594</v>
+        <v>sale_1791187181909</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C10" t="str">
-        <v>+92 339 8895511</v>
+        <v>+92 319 5466691</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Muse AI</v>
+        <v>Gemini Pro</v>
       </c>
       <c r="F10" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G10" t="str">
         <v>NA</v>
       </c>
       <c r="H10" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>18 Months (540 Days)</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="J10">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="K10" t="str">
         <v>Paid</v>
       </c>
       <c r="L10" t="str">
-        <v>2026-10-31</v>
+        <v>2028-03-27</v>
       </c>
       <c r="M10" t="str">
         <v/>
       </c>
       <c r="N10" t="str">
-        <v>2026-10-02T15:18:35.594Z</v>
+        <v>2026-10-05T07:59:41.909Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>sale_1790946519871</v>
+        <v>sale_1791184673171</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C11" t="str">
-        <v>+92 337 4695990</v>
+        <v>+92 303 5733146</v>
       </c>
       <c r="D11" t="str">
         <v/>
       </c>
       <c r="E11" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F11" t="str">
         <v>Private</v>
@@ -864,80 +863,80 @@
         <v>NA</v>
       </c>
       <c r="H11" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="K11" t="str">
         <v>Paid</v>
       </c>
       <c r="L11" t="str">
-        <v>2026-12-30</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M11" t="str">
         <v/>
       </c>
       <c r="N11" t="str">
-        <v>2026-10-02T13:08:39.871Z</v>
+        <v>2026-10-05T07:17:53.172Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sale_1790946456992</v>
+        <v>sale_1791183478163</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C12" t="str">
-        <v>+92 310 8747472</v>
+        <v>3425091286</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F12" t="str">
         <v>Shared</v>
       </c>
       <c r="G12" t="str">
-        <v>nor8@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H12" t="str">
-        <v>6 Months (180 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="K12" t="str">
         <v>Paid</v>
       </c>
       <c r="L12" t="str">
-        <v>2027-03-30</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M12" t="str">
         <v/>
       </c>
       <c r="N12" t="str">
-        <v>2026-10-02T13:07:36.993Z</v>
+        <v>2026-10-05T06:57:58.163Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sale_1790941037212</v>
+        <v>sale_1791183466887</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C13" t="str">
-        <v>30474552522</v>
+        <v>3199182226</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -949,7 +948,7 @@
         <v>Shared</v>
       </c>
       <c r="G13" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H13" t="str">
         <v>1 Month (30 Days)</v>
@@ -964,156 +963,156 @@
         <v>Paid</v>
       </c>
       <c r="L13" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-03</v>
       </c>
       <c r="M13" t="str">
         <v/>
       </c>
       <c r="N13" t="str">
-        <v>2026-10-02T11:37:17.212Z</v>
+        <v>2026-10-05T06:57:46.887Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sale_1790940354053</v>
+        <v>sale_1791153252198</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C14" t="str">
-        <v>+92 333 5598645</v>
+        <v>+92 326 7000168</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
       <c r="E14" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F14" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G14" t="str">
-        <v>alissaturner822@gmail.com</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H14" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14">
-        <v>1600</v>
+        <v>500</v>
       </c>
       <c r="K14" t="str">
         <v>Paid</v>
       </c>
       <c r="L14" t="str">
-        <v>2026-11-30</v>
+        <v>2027-01-02</v>
       </c>
       <c r="M14" t="str">
         <v/>
       </c>
       <c r="N14" t="str">
-        <v>2026-10-02T11:25:54.053Z</v>
+        <v>2026-10-04T22:34:12.198Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sale_1790939431495</v>
+        <v>sale_1791138731891</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C15" t="str">
-        <v>+92 301 2553778</v>
+        <v>+92 309 6116899</v>
       </c>
       <c r="D15" t="str">
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>Muse AI</v>
+        <v>Gemini Pro</v>
       </c>
       <c r="F15" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G15" t="str">
         <v>NA</v>
       </c>
       <c r="H15" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>18 Months (540 Days)</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="J15">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="K15" t="str">
         <v>Paid</v>
       </c>
       <c r="L15" t="str">
-        <v>2026-10-31</v>
+        <v>2028-03-26</v>
       </c>
       <c r="M15" t="str">
         <v/>
       </c>
       <c r="N15" t="str">
-        <v>2026-10-02T11:10:31.495Z</v>
+        <v>2026-10-04T18:32:11.892Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>sale_1790936221232</v>
+        <v>sale_1791137994648</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C16" t="str">
-        <v>3362088885</v>
+        <v>+92 302 4827701</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Surfshark</v>
+        <v>Gemini Pro</v>
       </c>
       <c r="F16" t="str">
         <v>Shared</v>
       </c>
       <c r="G16" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H16" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>18 Months (540 Days)</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="J16">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="K16" t="str">
         <v>Paid</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-10-31</v>
+        <v>2028-03-26</v>
       </c>
       <c r="M16" t="str">
         <v/>
       </c>
       <c r="N16" t="str">
-        <v>2026-10-02T10:17:01.232Z</v>
+        <v>2026-10-04T18:19:54.648Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>sale_1790934819273</v>
+        <v>sale_1791136834025</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C17" t="str">
-        <v>3362088885</v>
+        <v>3126811828</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -1125,7 +1124,7 @@
         <v>Shared</v>
       </c>
       <c r="G17" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H17" t="str">
         <v>1 Month (30 Days)</v>
@@ -1140,156 +1139,156 @@
         <v>Paid</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-02</v>
       </c>
       <c r="M17" t="str">
         <v/>
       </c>
       <c r="N17" t="str">
-        <v>2026-10-02T09:53:39.274Z</v>
+        <v>2026-10-04T18:00:34.025Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>sale_1790934132194</v>
+        <v>sale_1791136775857</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C18" t="str">
-        <v>3171626906</v>
+        <v>+92 311 7274561</v>
       </c>
       <c r="D18" t="str">
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F18" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G18" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>n</v>
       </c>
       <c r="H18" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I18">
         <v>1</v>
       </c>
       <c r="J18">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="K18" t="str">
         <v>Paid</v>
       </c>
       <c r="L18" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-02</v>
       </c>
       <c r="M18" t="str">
         <v/>
       </c>
       <c r="N18" t="str">
-        <v>2026-10-02T09:42:12.194Z</v>
+        <v>2026-10-04T17:59:35.857Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>sale_1790929984076</v>
+        <v>sale_1791136760132</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C19" t="str">
-        <v>3425091286</v>
+        <v>+92 308 5413116</v>
       </c>
       <c r="D19" t="str">
         <v/>
       </c>
       <c r="E19" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F19" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G19" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H19" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I19">
         <v>1</v>
       </c>
       <c r="J19">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="K19" t="str">
         <v>Paid</v>
       </c>
       <c r="L19" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-02</v>
       </c>
       <c r="M19" t="str">
         <v/>
       </c>
       <c r="N19" t="str">
-        <v>2026-10-02T08:33:04.076Z</v>
+        <v>2026-10-04T17:59:20.132Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>sale_1790928896570</v>
+        <v>sale_1791134215437</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C20" t="str">
-        <v>+92 335 9333443</v>
+        <v>3157839993</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F20" t="str">
         <v>Shared</v>
       </c>
       <c r="G20" t="str">
-        <v>NA</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H20" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>12 Months (360 Days)</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J20">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="K20" t="str">
         <v>Paid</v>
       </c>
       <c r="L20" t="str">
-        <v>2026-10-31</v>
+        <v>2027-09-28</v>
       </c>
       <c r="M20" t="str">
         <v/>
       </c>
       <c r="N20" t="str">
-        <v>2026-10-02T08:14:56.570Z</v>
+        <v>2026-10-04T17:16:55.437Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>sale_1790927823366</v>
+        <v>sale_1791106255456</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C21" t="str">
-        <v>3424112890 - 178132</v>
+        <v>971558178928</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -1301,39 +1300,39 @@
         <v>Shared</v>
       </c>
       <c r="G21" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H21" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J21">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="K21" t="str">
         <v>Paid</v>
       </c>
       <c r="L21" t="str">
-        <v>2026-10-31</v>
+        <v>2027-01-01</v>
       </c>
       <c r="M21" t="str">
         <v/>
       </c>
       <c r="N21" t="str">
-        <v>2026-10-02T07:57:03.366Z</v>
+        <v>2026-10-04T09:30:55.457Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>sale_1790927720999</v>
+        <v>sale_1791103826297</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C22" t="str">
-        <v>3355060692</v>
+        <v>3006831690</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -1345,39 +1344,39 @@
         <v>Shared</v>
       </c>
       <c r="G22" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H22" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>12 Months (360 Days)</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J22">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="K22" t="str">
         <v>Paid</v>
       </c>
       <c r="L22" t="str">
-        <v>2026-10-31</v>
+        <v>2027-09-28</v>
       </c>
       <c r="M22" t="str">
         <v/>
       </c>
       <c r="N22" t="str">
-        <v>2026-10-02T07:55:20.999Z</v>
+        <v>2026-10-04T08:50:26.297Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>sale_1790927520048</v>
+        <v>sale_1791102228323</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C23" t="str">
-        <v>3237432065</v>
+        <v>3047732450</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -1389,39 +1388,39 @@
         <v>Shared</v>
       </c>
       <c r="G23" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>abd151@kuromee.com</v>
       </c>
       <c r="H23" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>12 Months (360 Days)</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="J23">
-        <v>400</v>
+        <v>1400</v>
       </c>
       <c r="K23" t="str">
         <v>Paid</v>
       </c>
       <c r="L23" t="str">
-        <v>2026-11-30</v>
+        <v>2027-09-28</v>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v>2026-10-02T07:52:00.048Z</v>
+        <v>2026-10-04T08:23:48.324Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>sale_1790927399372</v>
+        <v>sale_1791099523357</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C24" t="str">
-        <v>3226763778</v>
+        <v>3081503007</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -1448,24 +1447,24 @@
         <v>Paid</v>
       </c>
       <c r="L24" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-02</v>
       </c>
       <c r="M24" t="str">
         <v/>
       </c>
       <c r="N24" t="str">
-        <v>2026-10-02T07:49:59.372Z</v>
+        <v>2026-10-04T07:38:43.357Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>sale_1790927194315</v>
+        <v>sale_1791098261508</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C25" t="str">
-        <v>3087182016</v>
+        <v>3007034330</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -1480,124 +1479,124 @@
         <v>abd150@kuromee.com</v>
       </c>
       <c r="H25" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="K25" t="str">
         <v>Paid</v>
       </c>
       <c r="L25" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-02</v>
       </c>
       <c r="M25" t="str">
         <v/>
       </c>
       <c r="N25" t="str">
-        <v>2026-10-02T07:46:34.315Z</v>
+        <v>2026-10-04T07:17:41.508Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>sale_1790926790421</v>
+        <v>sale_1791064529531</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C26" t="str">
-        <v>3424112890 - 161547</v>
+        <v>+92 302 7283125</v>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F26" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G26" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H26" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I26">
         <v>1</v>
       </c>
       <c r="J26">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="K26" t="str">
         <v>Paid</v>
       </c>
       <c r="L26" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M26" t="str">
         <v/>
       </c>
       <c r="N26" t="str">
-        <v>2026-10-02T07:39:50.422Z</v>
+        <v>2026-10-03T21:55:29.531Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>sale_1790890878620</v>
+        <v>sale_1791064497321</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C27" t="str">
-        <v>3336677666</v>
+        <v>+92 300 6831690</v>
       </c>
       <c r="D27" t="str">
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F27" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G27" t="str">
-        <v>abd150@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H27" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I27">
         <v>1</v>
       </c>
       <c r="J27">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="K27" t="str">
         <v>Paid</v>
       </c>
       <c r="L27" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M27" t="str">
         <v/>
       </c>
       <c r="N27" t="str">
-        <v>2026-10-01T21:41:18.621Z</v>
+        <v>2026-10-03T21:54:57.321Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>sale_1790889330982</v>
+        <v>sale_1791037027100</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C28" t="str">
-        <v>+92 333 7180888</v>
+        <v>+92 309 3030483</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -1612,80 +1611,80 @@
         <v>NA</v>
       </c>
       <c r="H28" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I28">
         <v>1</v>
       </c>
       <c r="J28">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="K28" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L28" t="str">
-        <v>2026-10-31</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>2026-10-01T21:15:30.982Z</v>
+        <v>2026-10-03T14:17:07.100Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>sale_1790889019841</v>
+        <v>sale_1791036095236</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C29" t="str">
-        <v>+92 324 3715759</v>
+        <v>3413317078</v>
       </c>
       <c r="D29" t="str">
         <v/>
       </c>
       <c r="E29" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F29" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G29" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H29" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="K29" t="str">
         <v>Paid</v>
       </c>
       <c r="L29" t="str">
-        <v>2026-10-31</v>
+        <v>2026-12-01</v>
       </c>
       <c r="M29" t="str">
         <v/>
       </c>
       <c r="N29" t="str">
-        <v>2026-10-01T21:10:19.841Z</v>
+        <v>2026-10-03T14:01:35.236Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>sale_1790889206450</v>
+        <v>sale_1791035943610</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C30" t="str">
-        <v>447348556756 - 2 Devices</v>
+        <v>3158206979</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -1697,7 +1696,7 @@
         <v>Shared</v>
       </c>
       <c r="G30" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H30" t="str">
         <v>1 Month (30 Days)</v>
@@ -1706,30 +1705,30 @@
         <v>1</v>
       </c>
       <c r="J30">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K30" t="str">
         <v>Paid</v>
       </c>
       <c r="L30" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M30" t="str">
         <v/>
       </c>
       <c r="N30" t="str">
-        <v>2026-10-01T21:13:26.450Z</v>
+        <v>2026-10-03T13:59:03.610Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>sale_1790889149110</v>
+        <v>sale_1791035347968</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C31" t="str">
-        <v>3716928959</v>
+        <v>3091259797</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -1741,227 +1740,227 @@
         <v>Shared</v>
       </c>
       <c r="G31" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H31" t="str">
-        <v>2 Months (60 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="K31" t="str">
         <v>Paid</v>
       </c>
       <c r="L31" t="str">
-        <v>2026-11-29</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
-        <v>2026-10-01T21:12:29.110Z</v>
+        <v>2026-10-03T13:49:07.968Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>sale_1790888980587</v>
+        <v>sale_1791035307158</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C32" t="str">
-        <v>+92 337 8569003</v>
+        <v>3241266815</v>
       </c>
       <c r="D32" t="str">
         <v/>
       </c>
       <c r="E32" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F32" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G32" t="str">
-        <v>padmahastuti3@akunku.site|masuk123</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H32" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>3 Months (90 Days)</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J32">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="K32" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L32" t="str">
-        <v>2026-10-30</v>
+        <v>2026-12-31</v>
       </c>
       <c r="M32" t="str">
         <v/>
       </c>
       <c r="N32" t="str">
-        <v>2026-10-01T21:09:40.587Z</v>
+        <v>2026-10-03T13:48:27.158Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>sale_1790888790593</v>
+        <v>sale_1791035284989</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C33" t="str">
-        <v>+92 318 8934627</v>
+        <v>+92 314 7659690</v>
       </c>
       <c r="D33" t="str">
         <v/>
       </c>
       <c r="E33" t="str">
-        <v>Muse AI</v>
+        <v>CapCut</v>
       </c>
       <c r="F33" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G33" t="str">
-        <v>NA</v>
+        <v>jinawidamanik6@ccpro.id|masuk123</v>
       </c>
       <c r="H33" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month (25 Days)</v>
       </c>
       <c r="I33">
         <v>1</v>
       </c>
       <c r="J33">
-        <v>1200</v>
+        <v>550</v>
       </c>
       <c r="K33" t="str">
         <v>Paid</v>
       </c>
       <c r="L33" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M33" t="str">
         <v/>
       </c>
       <c r="N33" t="str">
-        <v>2026-10-01T21:06:30.593Z</v>
+        <v>2026-10-03T13:48:04.990Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>sale_1790888748366</v>
+        <v>sale_1791028064145</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C34" t="str">
-        <v>3121600439</v>
+        <v>+92 342 9665704</v>
       </c>
       <c r="D34" t="str">
         <v/>
       </c>
       <c r="E34" t="str">
-        <v>Surfshark</v>
+        <v>CapCut</v>
       </c>
       <c r="F34" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G34" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H34" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month (25 Days)</v>
       </c>
       <c r="I34">
         <v>1</v>
       </c>
       <c r="J34">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="K34" t="str">
         <v>Paid</v>
       </c>
       <c r="L34" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M34" t="str">
-        <v/>
+        <v>arthurwestbrook00q61@klingaii.com Capcut#1122</v>
       </c>
       <c r="N34" t="str">
-        <v>2026-10-01T21:05:48.366Z</v>
+        <v>2026-10-03T11:47:44.145Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>sale_1790888549930</v>
+        <v>sale_1791024242646</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C35" t="str">
-        <v>3148646368</v>
+        <v>+92 319 5466691</v>
       </c>
       <c r="D35" t="str">
         <v/>
       </c>
       <c r="E35" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F35" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G35" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H35" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>1 Month(s)</v>
       </c>
       <c r="I35">
         <v>1</v>
       </c>
       <c r="J35">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="K35" t="str">
         <v>Paid</v>
       </c>
       <c r="L35" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-01</v>
       </c>
       <c r="M35" t="str">
         <v/>
       </c>
       <c r="N35" t="str">
-        <v>2026-10-01T21:02:29.930Z</v>
+        <v>2026-10-03T10:44:02.646Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>sale_1790888489800</v>
+        <v>sale_1790972901458</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C36" t="str">
-        <v>3043943233 - 2 devices</v>
+        <v>+92 333 3707266</v>
       </c>
       <c r="D36" t="str">
         <v/>
       </c>
       <c r="E36" t="str">
-        <v>Surfshark</v>
+        <v>Nord</v>
       </c>
       <c r="F36" t="str">
         <v>Shared</v>
       </c>
       <c r="G36" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>nord9@kuromee.com</v>
       </c>
       <c r="H36" t="str">
         <v>3 Months (90 Days)</v>
@@ -1970,30 +1969,30 @@
         <v>3</v>
       </c>
       <c r="J36">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="K36" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L36" t="str">
-        <v>2026-12-29</v>
+        <v>2026-12-31</v>
       </c>
       <c r="M36" t="str">
-        <v>Payment 5 Oct</v>
+        <v/>
       </c>
       <c r="N36" t="str">
-        <v>2026-10-01T21:01:29.800Z</v>
+        <v>2026-10-02T20:28:21.458Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>sale_1790888426010</v>
+        <v>sale_1790971693632</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C37" t="str">
-        <v>3125698180</v>
+        <v>3038522190</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -2005,7 +2004,7 @@
         <v>Shared</v>
       </c>
       <c r="G37" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H37" t="str">
         <v>2 Months (60 Days)</v>
@@ -2017,27 +2016,27 @@
         <v>400</v>
       </c>
       <c r="K37" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L37" t="str">
-        <v>2026-11-29</v>
+        <v>2026-12-01</v>
       </c>
       <c r="M37" t="str">
-        <v>Payment Sunday 4 Oct</v>
+        <v/>
       </c>
       <c r="N37" t="str">
-        <v>2026-10-01T21:00:26.011Z</v>
+        <v>2026-10-02T20:08:13.632Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>sale_1790888378017</v>
+        <v>sale_1790967903952</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C38" t="str">
-        <v>3208546164</v>
+        <v>3452401920</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -2049,7 +2048,7 @@
         <v>Shared</v>
       </c>
       <c r="G38" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H38" t="str">
         <v>2 Months (60 Days)</v>
@@ -2064,24 +2063,24 @@
         <v>Paid</v>
       </c>
       <c r="L38" t="str">
-        <v>2026-11-29</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M38" t="str">
         <v/>
       </c>
       <c r="N38" t="str">
-        <v>2026-10-01T20:59:38.017Z</v>
+        <v>2026-10-02T19:05:03.952Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>sale_1790888324786</v>
+        <v>sale_1790966446338</v>
       </c>
       <c r="B39" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C39" t="str">
-        <v>3424112890 - 232013</v>
+        <v>3162936885</v>
       </c>
       <c r="D39" t="str">
         <v/>
@@ -2093,7 +2092,7 @@
         <v>Shared</v>
       </c>
       <c r="G39" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H39" t="str">
         <v>1 Month (30 Days)</v>
@@ -2108,36 +2107,36 @@
         <v>Paid</v>
       </c>
       <c r="L39" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M39" t="str">
         <v/>
       </c>
       <c r="N39" t="str">
-        <v>2026-10-01T20:58:44.786Z</v>
+        <v>2026-10-02T18:40:46.338Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>sale_1790871288858</v>
+        <v>sale_1790964840039</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C40" t="str">
-        <v>+92 336 6331621</v>
+        <v>3068258151</v>
       </c>
       <c r="D40" t="str">
         <v/>
       </c>
       <c r="E40" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F40" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G40" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H40" t="str">
         <v>1 Month (30 Days)</v>
@@ -2146,74 +2145,74 @@
         <v>1</v>
       </c>
       <c r="J40">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="K40" t="str">
         <v>Paid</v>
       </c>
       <c r="L40" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M40" t="str">
         <v/>
       </c>
       <c r="N40" t="str">
-        <v>2026-10-01T16:14:48.858Z</v>
+        <v>2026-10-02T18:14:00.039Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>sale_1790871264002</v>
+        <v>sale_1790964482569</v>
       </c>
       <c r="B41" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C41" t="str">
-        <v>+98 901 603 6081</v>
+        <v>+92 334 7132394</v>
       </c>
       <c r="D41" t="str">
         <v/>
       </c>
       <c r="E41" t="str">
-        <v>Nord</v>
+        <v>Muse AI</v>
       </c>
       <c r="F41" t="str">
         <v>Shared</v>
       </c>
       <c r="G41" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H41" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J41">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="K41" t="str">
         <v>Paid</v>
       </c>
       <c r="L41" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M41" t="str">
         <v/>
       </c>
       <c r="N41" t="str">
-        <v>2026-10-01T16:14:24.002Z</v>
+        <v>2026-10-02T18:08:02.570Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>sale_1790868862060</v>
+        <v>sale_1790964455099</v>
       </c>
       <c r="B42" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C42" t="str">
-        <v>+92 341 9010662</v>
+        <v>+92 318 8934627</v>
       </c>
       <c r="D42" t="str">
         <v/>
@@ -2222,7 +2221,7 @@
         <v>Muse AI</v>
       </c>
       <c r="F42" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G42" t="str">
         <v>NA</v>
@@ -2240,112 +2239,112 @@
         <v>Paid</v>
       </c>
       <c r="L42" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M42" t="str">
         <v/>
       </c>
       <c r="N42" t="str">
-        <v>2026-10-01T15:34:22.075Z</v>
+        <v>2026-10-02T18:07:35.099Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>sale_1790864924575</v>
+        <v>sale_1790955121286</v>
       </c>
       <c r="B43" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C43" t="str">
-        <v>+92 313 6762957</v>
+        <v>3424112890 - 810813</v>
       </c>
       <c r="D43" t="str">
         <v/>
       </c>
       <c r="E43" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F43" t="str">
         <v>Shared</v>
       </c>
       <c r="G43" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H43" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J43">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="K43" t="str">
-        <v>Paid</v>
+        <v>Pending</v>
       </c>
       <c r="L43" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M43" t="str">
         <v/>
       </c>
       <c r="N43" t="str">
-        <v>2026-10-01T14:28:44.576Z</v>
+        <v>2026-10-02T15:32:01.286Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>sale_1790864890520</v>
+        <v>sale_1790954315594</v>
       </c>
       <c r="B44" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C44" t="str">
-        <v>3166729551</v>
+        <v>+92 339 8895511</v>
       </c>
       <c r="D44" t="str">
         <v/>
       </c>
       <c r="E44" t="str">
-        <v>Surfshark</v>
+        <v>Muse AI</v>
       </c>
       <c r="F44" t="str">
         <v>Shared</v>
       </c>
       <c r="G44" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H44" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J44">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="K44" t="str">
         <v>Paid</v>
       </c>
       <c r="L44" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M44" t="str">
         <v/>
       </c>
       <c r="N44" t="str">
-        <v>2026-10-01T14:28:10.520Z</v>
+        <v>2026-10-02T15:18:35.594Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>sale_1790862744178</v>
+        <v>sale_1790946519871</v>
       </c>
       <c r="B45" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C45" t="str">
-        <v>+92 317 0295905</v>
+        <v>+92 337 4695990</v>
       </c>
       <c r="D45" t="str">
         <v/>
@@ -2354,10 +2353,10 @@
         <v>Nord</v>
       </c>
       <c r="F45" t="str">
-        <v>Shared</v>
+        <v>Private</v>
       </c>
       <c r="G45" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>NA</v>
       </c>
       <c r="H45" t="str">
         <v>3 Months (90 Days)</v>
@@ -2366,30 +2365,30 @@
         <v>3</v>
       </c>
       <c r="J45">
-        <v>600</v>
+        <v>1300</v>
       </c>
       <c r="K45" t="str">
         <v>Paid</v>
       </c>
       <c r="L45" t="str">
-        <v>2026-12-29</v>
+        <v>2026-12-30</v>
       </c>
       <c r="M45" t="str">
         <v/>
       </c>
       <c r="N45" t="str">
-        <v>2026-10-01T13:52:24.178Z</v>
+        <v>2026-10-02T13:08:39.871Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>sale_1790861118501</v>
+        <v>sale_1790946456992</v>
       </c>
       <c r="B46" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C46" t="str">
-        <v>+92 344 4643148</v>
+        <v>+92 310 8747472</v>
       </c>
       <c r="D46" t="str">
         <v/>
@@ -2401,51 +2400,51 @@
         <v>Shared</v>
       </c>
       <c r="G46" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>nor8@kuromee.com</v>
       </c>
       <c r="H46" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>6 Months (180 Days)</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="K46" t="str">
         <v>Paid</v>
       </c>
       <c r="L46" t="str">
-        <v>2026-12-29</v>
+        <v>2027-03-30</v>
       </c>
       <c r="M46" t="str">
         <v/>
       </c>
       <c r="N46" t="str">
-        <v>2026-10-01T13:25:18.501Z</v>
+        <v>2026-10-02T13:07:36.993Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>sale_1790853314445</v>
+        <v>sale_1790941037212</v>
       </c>
       <c r="B47" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C47" t="str">
-        <v>+92 302 7283125</v>
+        <v>30474552522</v>
       </c>
       <c r="D47" t="str">
         <v/>
       </c>
       <c r="E47" t="str">
-        <v>CapCut</v>
+        <v>Surfshark</v>
       </c>
       <c r="F47" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G47" t="str">
-        <v>NA</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H47" t="str">
         <v>1 Month (30 Days)</v>
@@ -2454,74 +2453,74 @@
         <v>1</v>
       </c>
       <c r="J47">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="K47" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L47" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M47" t="str">
-        <v>vukdsas@apricity.tech  masuk123</v>
+        <v/>
       </c>
       <c r="N47" t="str">
-        <v>2026-10-01T11:15:14.445Z</v>
+        <v>2026-10-02T11:37:17.212Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>sale_1790852538710</v>
+        <v>sale_1790940354053</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C48" t="str">
-        <v>+92 325 1501138</v>
+        <v>+92 333 5598645</v>
       </c>
       <c r="D48" t="str">
         <v/>
       </c>
       <c r="E48" t="str">
-        <v>Muse AI</v>
+        <v>Surfshark</v>
       </c>
       <c r="F48" t="str">
         <v>Private</v>
       </c>
       <c r="G48" t="str">
-        <v>N/A</v>
+        <v>alissaturner822@gmail.com</v>
       </c>
       <c r="H48" t="str">
-        <v>1 Month (30 Days)</v>
+        <v>2 Months (60 Days)</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J48">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="K48" t="str">
         <v>Paid</v>
       </c>
       <c r="L48" t="str">
-        <v>2026-10-30</v>
+        <v>2026-11-30</v>
       </c>
       <c r="M48" t="str">
         <v/>
       </c>
       <c r="N48" t="str">
-        <v>2026-10-01T11:02:18.710Z</v>
+        <v>2026-10-02T11:25:54.053Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>sale_1790852373016</v>
+        <v>sale_1790939431495</v>
       </c>
       <c r="B49" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C49" t="str">
-        <v>+92 301 7890066</v>
+        <v>+92 301 2553778</v>
       </c>
       <c r="D49" t="str">
         <v/>
@@ -2530,10 +2529,10 @@
         <v>Muse AI</v>
       </c>
       <c r="F49" t="str">
-        <v>Private</v>
+        <v>Shared</v>
       </c>
       <c r="G49" t="str">
-        <v>N/A</v>
+        <v>NA</v>
       </c>
       <c r="H49" t="str">
         <v>1 Month (30 Days)</v>
@@ -2542,30 +2541,30 @@
         <v>1</v>
       </c>
       <c r="J49">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="K49" t="str">
         <v>Paid</v>
       </c>
       <c r="L49" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M49" t="str">
         <v/>
       </c>
       <c r="N49" t="str">
-        <v>2026-10-01T10:59:33.016Z</v>
+        <v>2026-10-02T11:10:31.495Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>sale_1790850006978</v>
+        <v>sale_1790936221232</v>
       </c>
       <c r="B50" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C50" t="str">
-        <v>+92 342 4112890-534389</v>
+        <v>3362088885</v>
       </c>
       <c r="D50" t="str">
         <v/>
@@ -2577,7 +2576,7 @@
         <v>Shared</v>
       </c>
       <c r="G50" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H50" t="str">
         <v>1 Month (30 Days)</v>
@@ -2586,30 +2585,30 @@
         <v>1</v>
       </c>
       <c r="J50">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="K50" t="str">
         <v>Paid</v>
       </c>
       <c r="L50" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M50" t="str">
         <v/>
       </c>
       <c r="N50" t="str">
-        <v>2026-10-01T10:20:06.978Z</v>
+        <v>2026-10-02T10:17:01.232Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>sale_1790849948623</v>
+        <v>sale_1790934821042_1qpo</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C51" t="str">
-        <v>+92 349 6363398</v>
+        <v>3362088885</v>
       </c>
       <c r="D51" t="str">
         <v/>
@@ -2621,7 +2620,7 @@
         <v>Shared</v>
       </c>
       <c r="G51" t="str">
-        <v>abd149@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H51" t="str">
         <v>1 Month (30 Days)</v>
@@ -2636,201 +2635,1697 @@
         <v>Paid</v>
       </c>
       <c r="L51" t="str">
-        <v>2026-10-30</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M51" t="str">
         <v/>
       </c>
       <c r="N51" t="str">
-        <v>2026-10-01T10:19:08.625Z</v>
+        <v>2026-10-02T09:53:41.042Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>sale_1790844774858</v>
+        <v>sale_1790934819273</v>
       </c>
       <c r="B52" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C52" t="str">
-        <v>03035587360</v>
+        <v>3362088885</v>
       </c>
       <c r="D52" t="str">
         <v/>
       </c>
       <c r="E52" t="str">
-        <v>Gemini Pro</v>
+        <v>Surfshark</v>
       </c>
       <c r="F52" t="str">
         <v>Shared</v>
       </c>
       <c r="G52" t="str">
-        <v>Not applicable</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H52" t="str">
-        <v>18 Months (540 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I52">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J52">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K52" t="str">
         <v>Paid</v>
       </c>
       <c r="L52" t="str">
-        <v>2028-03-23</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M52" t="str">
         <v/>
       </c>
       <c r="N52" t="str">
-        <v>2026-10-01T08:52:54.860Z</v>
+        <v>2026-10-02T09:53:39.274Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>sale_1790841917101</v>
+        <v>sale_1790934132194</v>
       </c>
       <c r="B53" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C53" t="str">
-        <v>+92 340 7317084</v>
+        <v>3171626906</v>
       </c>
       <c r="D53" t="str">
         <v/>
       </c>
       <c r="E53" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F53" t="str">
         <v>Shared</v>
       </c>
       <c r="G53" t="str">
-        <v>nord9@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H53" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I53">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J53">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K53" t="str">
         <v>Paid</v>
       </c>
       <c r="L53" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M53" t="str">
         <v/>
       </c>
       <c r="N53" t="str">
-        <v>2026-10-01T08:05:17.101Z</v>
+        <v>2026-10-02T09:42:12.194Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>sale_1790839031379</v>
+        <v>sale_1790929984076</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C54" t="str">
-        <v>+92 340 7317084</v>
+        <v>3425091286</v>
       </c>
       <c r="D54" t="str">
         <v/>
       </c>
       <c r="E54" t="str">
-        <v>Nord</v>
+        <v>Surfshark</v>
       </c>
       <c r="F54" t="str">
         <v>Shared</v>
       </c>
       <c r="G54" t="str">
-        <v>Nord9@kuromee.com</v>
+        <v>abd150@kuromee.com</v>
       </c>
       <c r="H54" t="str">
-        <v>3 Months (90 Days)</v>
+        <v>1 Month (30 Days)</v>
       </c>
       <c r="I54">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J54">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K54" t="str">
         <v>Paid</v>
       </c>
       <c r="L54" t="str">
-        <v>2026-12-29</v>
+        <v>2026-10-31</v>
       </c>
       <c r="M54" t="str">
         <v/>
       </c>
       <c r="N54" t="str">
-        <v>2026-10-01T07:17:11.379Z</v>
+        <v>2026-10-02T08:33:04.076Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>sale_1790838846301</v>
+        <v>sale_1790928896570</v>
       </c>
       <c r="B55" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C55" t="str">
+        <v>+92 335 9333443</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G55" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H55" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I55">
+        <v>1</v>
+      </c>
+      <c r="J55">
+        <v>1500</v>
+      </c>
+      <c r="K55" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L55" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M55" t="str">
+        <v/>
+      </c>
+      <c r="N55" t="str">
+        <v>2026-10-02T08:14:56.570Z</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>sale_1790927823366</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C56" t="str">
+        <v>3424112890 - 178132</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G56" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H56" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I56">
+        <v>1</v>
+      </c>
+      <c r="J56">
+        <v>200</v>
+      </c>
+      <c r="K56" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L56" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M56" t="str">
+        <v/>
+      </c>
+      <c r="N56" t="str">
+        <v>2026-10-02T07:57:03.366Z</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>sale_1790927720999</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C57" t="str">
+        <v>3355060692</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G57" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H57" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I57">
+        <v>1</v>
+      </c>
+      <c r="J57">
+        <v>250</v>
+      </c>
+      <c r="K57" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L57" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M57" t="str">
+        <v/>
+      </c>
+      <c r="N57" t="str">
+        <v>2026-10-02T07:55:20.999Z</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>sale_1790927520048</v>
+      </c>
+      <c r="B58" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C58" t="str">
+        <v>3237432065</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G58" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H58" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="I58">
+        <v>2</v>
+      </c>
+      <c r="J58">
+        <v>400</v>
+      </c>
+      <c r="K58" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L58" t="str">
+        <v>2026-11-30</v>
+      </c>
+      <c r="M58" t="str">
+        <v/>
+      </c>
+      <c r="N58" t="str">
+        <v>2026-10-02T07:52:00.048Z</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>sale_1790927399372</v>
+      </c>
+      <c r="B59" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C59" t="str">
+        <v>3226763778</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G59" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H59" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I59">
+        <v>1</v>
+      </c>
+      <c r="J59">
+        <v>250</v>
+      </c>
+      <c r="K59" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L59" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M59" t="str">
+        <v/>
+      </c>
+      <c r="N59" t="str">
+        <v>2026-10-02T07:49:59.372Z</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>sale_1790927194315</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C60" t="str">
+        <v>3087182016</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G60" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H60" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I60">
+        <v>1</v>
+      </c>
+      <c r="J60">
+        <v>250</v>
+      </c>
+      <c r="K60" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L60" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M60" t="str">
+        <v/>
+      </c>
+      <c r="N60" t="str">
+        <v>2026-10-02T07:46:34.315Z</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>sale_1790926790421</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C61" t="str">
+        <v>3424112890 - 161547</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G61" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H61" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61">
+        <v>200</v>
+      </c>
+      <c r="K61" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L61" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M61" t="str">
+        <v/>
+      </c>
+      <c r="N61" t="str">
+        <v>2026-10-02T07:39:50.422Z</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>sale_1790890878620</v>
+      </c>
+      <c r="B62" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C62" t="str">
+        <v>3336677666</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G62" t="str">
+        <v>abd150@kuromee.com</v>
+      </c>
+      <c r="H62" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I62">
+        <v>1</v>
+      </c>
+      <c r="J62">
+        <v>250</v>
+      </c>
+      <c r="K62" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L62" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M62" t="str">
+        <v/>
+      </c>
+      <c r="N62" t="str">
+        <v>2026-10-01T21:41:18.621Z</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>sale_1790889330982</v>
+      </c>
+      <c r="B63" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C63" t="str">
+        <v>+92 333 7180888</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G63" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H63" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I63">
+        <v>1</v>
+      </c>
+      <c r="J63">
+        <v>1000</v>
+      </c>
+      <c r="K63" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L63" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M63" t="str">
+        <v/>
+      </c>
+      <c r="N63" t="str">
+        <v>2026-10-01T21:15:30.982Z</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>sale_1790889019841</v>
+      </c>
+      <c r="B64" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C64" t="str">
+        <v>+92 324 3715759</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G64" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H64" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I64">
+        <v>1</v>
+      </c>
+      <c r="J64">
+        <v>1000</v>
+      </c>
+      <c r="K64" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L64" t="str">
+        <v>2026-10-31</v>
+      </c>
+      <c r="M64" t="str">
+        <v/>
+      </c>
+      <c r="N64" t="str">
+        <v>2026-10-01T21:10:19.841Z</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>sale_1790889206450</v>
+      </c>
+      <c r="B65" t="str">
         <v>2026-10-01</v>
       </c>
-      <c r="C55" t="str">
-        <v>3085352533</v>
-      </c>
-      <c r="D55" t="str">
-        <v/>
-      </c>
-      <c r="E55" t="str">
+      <c r="C65" t="str">
+        <v>447348556756 - 2 Devices</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
         <v>Surfshark</v>
       </c>
-      <c r="F55" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="G55" t="str">
+      <c r="F65" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G65" t="str">
         <v>abd149@kuromee.com</v>
       </c>
-      <c r="H55" t="str">
+      <c r="H65" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I65">
+        <v>1</v>
+      </c>
+      <c r="J65">
+        <v>500</v>
+      </c>
+      <c r="K65" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L65" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M65" t="str">
+        <v/>
+      </c>
+      <c r="N65" t="str">
+        <v>2026-10-01T21:13:26.450Z</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>sale_1790889149110</v>
+      </c>
+      <c r="B66" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C66" t="str">
+        <v>3716928959</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G66" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H66" t="str">
         <v>2 Months (60 Days)</v>
       </c>
-      <c r="I55">
+      <c r="I66">
         <v>2</v>
       </c>
-      <c r="J55">
-        <v>800</v>
-      </c>
-      <c r="K55" t="str">
+      <c r="J66">
+        <v>400</v>
+      </c>
+      <c r="K66" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L66" t="str">
+        <v>2026-11-29</v>
+      </c>
+      <c r="M66" t="str">
+        <v/>
+      </c>
+      <c r="N66" t="str">
+        <v>2026-10-01T21:12:29.110Z</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>sale_1790888980587</v>
+      </c>
+      <c r="B67" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C67" t="str">
+        <v>+92 337 8569003</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G67" t="str">
+        <v>padmahastuti3@akunku.site|masuk123</v>
+      </c>
+      <c r="H67" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I67">
+        <v>1</v>
+      </c>
+      <c r="J67">
+        <v>750</v>
+      </c>
+      <c r="K67" t="str">
         <v>Pending</v>
       </c>
-      <c r="L55" t="str">
+      <c r="L67" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M67" t="str">
+        <v/>
+      </c>
+      <c r="N67" t="str">
+        <v>2026-10-01T21:09:40.587Z</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>sale_1790888790593</v>
+      </c>
+      <c r="B68" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C68" t="str">
+        <v>+92 318 8934627</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G68" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H68" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I68">
+        <v>1</v>
+      </c>
+      <c r="J68">
+        <v>1200</v>
+      </c>
+      <c r="K68" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L68" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M68" t="str">
+        <v/>
+      </c>
+      <c r="N68" t="str">
+        <v>2026-10-01T21:06:30.593Z</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>sale_1790888748366</v>
+      </c>
+      <c r="B69" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C69" t="str">
+        <v>3121600439</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G69" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H69" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I69">
+        <v>1</v>
+      </c>
+      <c r="J69">
+        <v>250</v>
+      </c>
+      <c r="K69" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L69" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M69" t="str">
+        <v/>
+      </c>
+      <c r="N69" t="str">
+        <v>2026-10-01T21:05:48.366Z</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>sale_1790888549930</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C70" t="str">
+        <v>3148646368</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G70" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H70" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I70">
+        <v>1</v>
+      </c>
+      <c r="J70">
+        <v>200</v>
+      </c>
+      <c r="K70" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L70" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M70" t="str">
+        <v/>
+      </c>
+      <c r="N70" t="str">
+        <v>2026-10-01T21:02:29.930Z</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>sale_1790888489800</v>
+      </c>
+      <c r="B71" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C71" t="str">
+        <v>3043943233 - 2 devices</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G71" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H71" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I71">
+        <v>3</v>
+      </c>
+      <c r="J71">
+        <v>1000</v>
+      </c>
+      <c r="K71" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L71" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M71" t="str">
+        <v>Payment 5 Oct</v>
+      </c>
+      <c r="N71" t="str">
+        <v>2026-10-01T21:01:29.800Z</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>sale_1790888426010</v>
+      </c>
+      <c r="B72" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C72" t="str">
+        <v>3125698180</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G72" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H72" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="I72">
+        <v>2</v>
+      </c>
+      <c r="J72">
+        <v>400</v>
+      </c>
+      <c r="K72" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L72" t="str">
         <v>2026-11-29</v>
       </c>
-      <c r="M55" t="str">
-        <v>2 Devices</v>
-      </c>
-      <c r="N55" t="str">
-        <v>2026-10-01T07:14:06.302Z</v>
+      <c r="M72" t="str">
+        <v>Payment Sunday 4 Oct</v>
+      </c>
+      <c r="N72" t="str">
+        <v>2026-10-01T21:00:26.011Z</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>sale_1790888378017</v>
+      </c>
+      <c r="B73" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C73" t="str">
+        <v>3208546164</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G73" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H73" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="I73">
+        <v>2</v>
+      </c>
+      <c r="J73">
+        <v>400</v>
+      </c>
+      <c r="K73" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L73" t="str">
+        <v>2026-11-29</v>
+      </c>
+      <c r="M73" t="str">
+        <v/>
+      </c>
+      <c r="N73" t="str">
+        <v>2026-10-01T20:59:38.017Z</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>sale_1790888324786</v>
+      </c>
+      <c r="B74" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C74" t="str">
+        <v>3424112890 - 232013</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G74" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H74" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I74">
+        <v>1</v>
+      </c>
+      <c r="J74">
+        <v>250</v>
+      </c>
+      <c r="K74" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L74" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M74" t="str">
+        <v/>
+      </c>
+      <c r="N74" t="str">
+        <v>2026-10-01T20:58:44.786Z</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>sale_1790871288858</v>
+      </c>
+      <c r="B75" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C75" t="str">
+        <v>+92 336 6331621</v>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G75" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H75" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I75">
+        <v>1</v>
+      </c>
+      <c r="J75">
+        <v>1200</v>
+      </c>
+      <c r="K75" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L75" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M75" t="str">
+        <v/>
+      </c>
+      <c r="N75" t="str">
+        <v>2026-10-01T16:14:48.858Z</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>sale_1790871264002</v>
+      </c>
+      <c r="B76" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C76" t="str">
+        <v>+98 901 603 6081</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G76" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H76" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I76">
+        <v>3</v>
+      </c>
+      <c r="J76">
+        <v>500</v>
+      </c>
+      <c r="K76" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L76" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M76" t="str">
+        <v/>
+      </c>
+      <c r="N76" t="str">
+        <v>2026-10-01T16:14:24.002Z</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>sale_1790868862060</v>
+      </c>
+      <c r="B77" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C77" t="str">
+        <v>+92 341 9010662</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G77" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H77" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I77">
+        <v>1</v>
+      </c>
+      <c r="J77">
+        <v>1000</v>
+      </c>
+      <c r="K77" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L77" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M77" t="str">
+        <v/>
+      </c>
+      <c r="N77" t="str">
+        <v>2026-10-01T15:34:22.075Z</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>sale_1790864924575</v>
+      </c>
+      <c r="B78" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C78" t="str">
+        <v>+92 313 6762957</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G78" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H78" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I78">
+        <v>3</v>
+      </c>
+      <c r="J78">
+        <v>500</v>
+      </c>
+      <c r="K78" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L78" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M78" t="str">
+        <v/>
+      </c>
+      <c r="N78" t="str">
+        <v>2026-10-01T14:28:44.576Z</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>sale_1790864890520</v>
+      </c>
+      <c r="B79" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C79" t="str">
+        <v>3166729551</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G79" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H79" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I79">
+        <v>3</v>
+      </c>
+      <c r="J79">
+        <v>600</v>
+      </c>
+      <c r="K79" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L79" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M79" t="str">
+        <v/>
+      </c>
+      <c r="N79" t="str">
+        <v>2026-10-01T14:28:10.520Z</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>sale_1790862744178</v>
+      </c>
+      <c r="B80" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C80" t="str">
+        <v>+92 317 0295905</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G80" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H80" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I80">
+        <v>3</v>
+      </c>
+      <c r="J80">
+        <v>600</v>
+      </c>
+      <c r="K80" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L80" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M80" t="str">
+        <v/>
+      </c>
+      <c r="N80" t="str">
+        <v>2026-10-01T13:52:24.178Z</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>sale_1790861118501</v>
+      </c>
+      <c r="B81" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C81" t="str">
+        <v>+92 344 4643148</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G81" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H81" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I81">
+        <v>3</v>
+      </c>
+      <c r="J81">
+        <v>500</v>
+      </c>
+      <c r="K81" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L81" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M81" t="str">
+        <v/>
+      </c>
+      <c r="N81" t="str">
+        <v>2026-10-01T13:25:18.501Z</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>sale_1790853314445</v>
+      </c>
+      <c r="B82" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C82" t="str">
+        <v>+92 302 7283125</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G82" t="str">
+        <v>NA</v>
+      </c>
+      <c r="H82" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I82">
+        <v>1</v>
+      </c>
+      <c r="J82">
+        <v>750</v>
+      </c>
+      <c r="K82" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L82" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M82" t="str">
+        <v>vukdsas@apricity.tech  masuk123</v>
+      </c>
+      <c r="N82" t="str">
+        <v>2026-10-01T11:15:14.445Z</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>sale_1790852538710</v>
+      </c>
+      <c r="B83" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C83" t="str">
+        <v>+92 325 1501138</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G83" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H83" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I83">
+        <v>1</v>
+      </c>
+      <c r="J83">
+        <v>1000</v>
+      </c>
+      <c r="K83" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L83" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M83" t="str">
+        <v/>
+      </c>
+      <c r="N83" t="str">
+        <v>2026-10-01T11:02:18.710Z</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>sale_1790852373016</v>
+      </c>
+      <c r="B84" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C84" t="str">
+        <v>+92 301 7890066</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Private</v>
+      </c>
+      <c r="G84" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H84" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I84">
+        <v>1</v>
+      </c>
+      <c r="J84">
+        <v>1500</v>
+      </c>
+      <c r="K84" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L84" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M84" t="str">
+        <v/>
+      </c>
+      <c r="N84" t="str">
+        <v>2026-10-01T10:59:33.016Z</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>sale_1790850006978</v>
+      </c>
+      <c r="B85" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C85" t="str">
+        <v>+92 342 4112890-534389</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G85" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H85" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I85">
+        <v>1</v>
+      </c>
+      <c r="J85">
+        <v>200</v>
+      </c>
+      <c r="K85" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L85" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M85" t="str">
+        <v/>
+      </c>
+      <c r="N85" t="str">
+        <v>2026-10-01T10:20:06.978Z</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>sale_1790849948623</v>
+      </c>
+      <c r="B86" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C86" t="str">
+        <v>+92 349 6363398</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G86" t="str">
+        <v>abd149@kuromee.com</v>
+      </c>
+      <c r="H86" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="I86">
+        <v>1</v>
+      </c>
+      <c r="J86">
+        <v>250</v>
+      </c>
+      <c r="K86" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L86" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="M86" t="str">
+        <v/>
+      </c>
+      <c r="N86" t="str">
+        <v>2026-10-01T10:19:08.625Z</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>sale_1790844774858</v>
+      </c>
+      <c r="B87" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C87" t="str">
+        <v>03035587360</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G87" t="str">
+        <v>Not applicable</v>
+      </c>
+      <c r="H87" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="I87">
+        <v>18</v>
+      </c>
+      <c r="J87">
+        <v>500</v>
+      </c>
+      <c r="K87" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L87" t="str">
+        <v>2028-03-23</v>
+      </c>
+      <c r="M87" t="str">
+        <v/>
+      </c>
+      <c r="N87" t="str">
+        <v>2026-10-01T08:52:54.860Z</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>sale_1790841917101</v>
+      </c>
+      <c r="B88" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C88" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G88" t="str">
+        <v>nord9@kuromee.com</v>
+      </c>
+      <c r="H88" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I88">
+        <v>3</v>
+      </c>
+      <c r="J88">
+        <v>500</v>
+      </c>
+      <c r="K88" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L88" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M88" t="str">
+        <v/>
+      </c>
+      <c r="N88" t="str">
+        <v>2026-10-01T08:05:17.101Z</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>sale_1790839031379</v>
+      </c>
+      <c r="B89" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C89" t="str">
+        <v>+92 340 7317084</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Nord9@kuromee.com</v>
+      </c>
+      <c r="H89" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="I89">
+        <v>3</v>
+      </c>
+      <c r="J89">
+        <v>500</v>
+      </c>
+      <c r="K89" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="L89" t="str">
+        <v>2026-12-29</v>
+      </c>
+      <c r="M89" t="str">
+        <v/>
+      </c>
+      <c r="N89" t="str">
+        <v>2026-10-01T07:17:11.379Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N89"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2854,444 +4349,187 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>exp_1790946533413</v>
+        <v>exp_1791205545999</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-05</v>
       </c>
       <c r="C2" t="str">
         <v>Vendor Purchasing</v>
       </c>
       <c r="D2" t="str">
-        <v>Nord purchasing</v>
+        <v>baktionopradana64@akunku.site|masuk123 qaoyxh@apricity.tech:masuk123</v>
       </c>
       <c r="E2">
-        <v>850</v>
+        <v>700</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-02T13:08:53.414Z</v>
+        <v>2026-10-05T13:05:45.999Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>exp_1790940392222</v>
+        <v>exp_1791035398823</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C3" t="str">
         <v>Vendor Purchasing</v>
       </c>
       <c r="D3" t="str">
-        <v>alissaturner822@gmail.com   Surfshark Private Payment</v>
+        <v>arthurwestbrook00q61@klingaii.com Capcut#1122</v>
       </c>
       <c r="E3">
-        <v>750</v>
+        <v>380</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-10-02T11:26:32.222Z</v>
+        <v>2026-10-03T13:49:58.823Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>exp_1790889252470</v>
+        <v>exp_1791035383336</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-03</v>
       </c>
       <c r="C4" t="str">
         <v>Vendor Purchasing</v>
       </c>
       <c r="D4" t="str">
-        <v>Surfshark/Nord Paid</v>
+        <v>jinawidamanik6@ccpro.id|masuk123</v>
       </c>
       <c r="E4">
-        <v>1600</v>
+        <v>350</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-10-01T21:14:12.470Z</v>
+        <v>2026-10-03T13:49:43.337Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>exp_1790888895390</v>
+        <v>exp_1791018590950</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C5" t="str">
-        <v>Vendor Purchasing</v>
+        <v>Meta Ads</v>
       </c>
       <c r="D5" t="str">
-        <v>Capcut padmahastuti3@akunku.site|masuk123</v>
+        <v>Meta Ads</v>
       </c>
       <c r="E5">
-        <v>350</v>
+        <v>2000</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-10-01T21:08:15.390Z</v>
+        <v>2026-10-03T09:09:50.950Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>exp_1790865001001</v>
+        <v>exp_1790940392222</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C6" t="str">
         <v>Vendor Purchasing</v>
       </c>
       <c r="D6" t="str">
-        <v>Capcut Account For Luxury online Store   vukdsas@apricity.tech:masuk123</v>
+        <v>alissaturner822@gmail.com   Surfshark Private Payment</v>
       </c>
       <c r="E6">
-        <v>350</v>
+        <v>750</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-10-01T14:30:01.001Z</v>
+        <v>2026-10-02T11:26:32.222Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>exp_1790810881227_1bq9</v>
+        <v>exp_1790889252470</v>
       </c>
       <c r="B7" t="str">
         <v>2026-10-01</v>
       </c>
       <c r="C7" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Surfshark/Nord Paid</v>
+      </c>
+      <c r="E7">
+        <v>1600</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-10-01T21:14:12.470Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>exp_1790888895390</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Capcut padmahastuti3@akunku.site|masuk123</v>
+      </c>
+      <c r="E8">
+        <v>350</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-10-01T21:08:15.390Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>exp_1790865001001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Vendor Purchasing</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Capcut Account For Luxury online Store   vukdsas@apricity.tech:masuk123</v>
+      </c>
+      <c r="E9">
+        <v>350</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-10-01T14:30:01.001Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>exp_1790810881227_1bq9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C10" t="str">
         <v>Meta Ads</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D10" t="str">
         <v>Meta Ads Campaign</v>
       </c>
-      <c r="E7">
+      <c r="E10">
         <v>500</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F10" t="str">
         <v>2026-09-30T23:28:01.227Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Product Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Account Type</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Plan Duration (Months)</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Plan Description</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Price (Rs.)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="str">
-        <v>1 Month (30 Days)</v>
-      </c>
-      <c r="E2">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2 Months (60 Days)</v>
-      </c>
-      <c r="E3">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4" t="str">
-        <v>3 Months (90 Days)</v>
-      </c>
-      <c r="E4">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="D5" t="str">
-        <v>6 Months (180 Days)</v>
-      </c>
-      <c r="E5">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C6">
-        <v>12</v>
-      </c>
-      <c r="D6" t="str">
-        <v>12 Months (360 Days)</v>
-      </c>
-      <c r="E6">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Private</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2 Months (60 Days)</v>
-      </c>
-      <c r="E7">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Surfshark</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Private</v>
-      </c>
-      <c r="C8">
-        <v>12</v>
-      </c>
-      <c r="D8" t="str">
-        <v>1 Year (360 Days)</v>
-      </c>
-      <c r="E8">
-        <v>9499</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C9">
-        <v>3</v>
-      </c>
-      <c r="D9" t="str">
-        <v>3 Months (90 Days)</v>
-      </c>
-      <c r="E9">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C10">
-        <v>6</v>
-      </c>
-      <c r="D10" t="str">
-        <v>6 Months (180 Days)</v>
-      </c>
-      <c r="E10">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C11">
-        <v>9</v>
-      </c>
-      <c r="D11" t="str">
-        <v>9 Months (270 Days)</v>
-      </c>
-      <c r="E11">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C12">
-        <v>12</v>
-      </c>
-      <c r="D12" t="str">
-        <v>12 Months (360 Days)</v>
-      </c>
-      <c r="E12">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Private</v>
-      </c>
-      <c r="C13">
-        <v>3</v>
-      </c>
-      <c r="D13" t="str">
-        <v>3 Months (90 Days)</v>
-      </c>
-      <c r="E13">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Nord</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Private</v>
-      </c>
-      <c r="C14">
-        <v>12</v>
-      </c>
-      <c r="D14" t="str">
-        <v>12 Months (360 Days)</v>
-      </c>
-      <c r="E14">
-        <v>6500</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Gemini Pro</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C15">
-        <v>18</v>
-      </c>
-      <c r="D15" t="str">
-        <v>18 Months (540 Days)</v>
-      </c>
-      <c r="E15">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>CapCut</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" t="str">
-        <v>1 Month (30 Days)</v>
-      </c>
-      <c r="E16">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" t="str">
-        <v>1 Month (30 Days)</v>
-      </c>
-      <c r="E17">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Muse AI</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Shared</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18" t="str">
-        <v>1 Month (30 Days)</v>
-      </c>
-      <c r="E18">
-        <v>500</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Connect live Upstash Redis cloud database for real-time mobile/laptop sync and add specific date sales section
</commit_message>
<xml_diff>
--- a/data/AB_Tools_Business_Ledger.xlsx
+++ b/data/AB_Tools_Business_Ledger.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Sales" sheetId="1" r:id="rId1"/>
     <sheet name="Expenses" sheetId="2" r:id="rId2"/>
+    <sheet name="Products" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -784,7 +785,7 @@
         <v>200</v>
       </c>
       <c r="K9" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="L9" t="str">
         <v>2026-11-03</v>
@@ -4532,4 +4533,355 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E20"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Product Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Account Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Plan Duration (Months)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Plan Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Price (Rs.)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="E2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="E3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="E4">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5" t="str">
+        <v>6 Months (180 Days)</v>
+      </c>
+      <c r="E5">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6" t="str">
+        <v>12 Months (360 Days)</v>
+      </c>
+      <c r="E6">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2 Months (60 Days)</v>
+      </c>
+      <c r="E7">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Surfshark</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8" t="str">
+        <v>1 Year (360 Days)</v>
+      </c>
+      <c r="E8">
+        <v>9499</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="E9">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10" t="str">
+        <v>6 Months (180 Days)</v>
+      </c>
+      <c r="E10">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C11">
+        <v>9</v>
+      </c>
+      <c r="D11" t="str">
+        <v>9 Months (270 Days)</v>
+      </c>
+      <c r="E11">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C12">
+        <v>12</v>
+      </c>
+      <c r="D12" t="str">
+        <v>12 Months (360 Days)</v>
+      </c>
+      <c r="E12">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13" t="str">
+        <v>3 Months (90 Days)</v>
+      </c>
+      <c r="E13">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Nord</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C14">
+        <v>12</v>
+      </c>
+      <c r="D14" t="str">
+        <v>12 Months (360 Days)</v>
+      </c>
+      <c r="E14">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C15">
+        <v>18</v>
+      </c>
+      <c r="D15" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="E15">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="str">
+        <v>1 Month (25 Days)</v>
+      </c>
+      <c r="E16">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>ChatGPT</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="str">
+        <v>1 Month (30 Days)</v>
+      </c>
+      <c r="E17">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Muse AI</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>1 Month(s)</v>
+      </c>
+      <c r="E18">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Gemini Pro</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19" t="str">
+        <v>18 Months (540 Days)</v>
+      </c>
+      <c r="E19">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>CapCut</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="str">
+        <v>1 Month (25 Days)</v>
+      </c>
+      <c r="E20">
+        <v>550</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>